<commit_message>
minor change in hazard file xlsx
</commit_message>
<xml_diff>
--- a/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/Input from Raghukanth/_fromSTGR_Modfied_HazardData_2026-08-18_sks_v1.xlsx
+++ b/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/Input from Raghukanth/_fromSTGR_Modfied_HazardData_2026-08-18_sks_v1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\OpenSees_PracticeExamples\ida-spo-msa\HazardAnalysis\gm-selection\2020_NBC_MyCopy_new-main\Input from Raghukanth\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psb\Downloads\GitHub\ida-spo-msa\HazardAnalysis\gm-selection\2020_NBC_MyCopy_new-main\Input from Raghukanth\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215D9562-71B9-4E48-A5A2-A2BE9FD300D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="844" activeTab="3"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="844" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HazCur-STGR-26-08-12" sheetId="1" r:id="rId1"/>
@@ -18,7 +19,7 @@
     <sheet name="Guwa-HazCur-STGR-26-08-18" sheetId="8" r:id="rId4"/>
     <sheet name="Delhi-HazCur-STGR-2026-08-18" sheetId="7" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -469,7 +470,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
@@ -1025,7 +1026,7 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1143,7 +1144,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
@@ -1169,7 +1169,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1189,12 +1189,8 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1226,6 +1222,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1262,12 +1264,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -9519,7 +9515,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-IN"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13396,7 +13392,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-IN"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13506,7 +13502,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-IN"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13687,7 +13683,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -17762,7 +17757,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -17884,7 +17878,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -19359,7 +19352,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -20217,7 +20209,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -21079,7 +21070,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -21941,7 +21931,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -30086,7 +30075,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A6C3C07-F93F-9F51-FDD5-3CF25350CC5E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -30958,7 +30947,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEB8AC6E-3D40-786B-9734-82A31A53DB42}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -30999,7 +30988,7 @@
         <xdr:cNvPr id="2" name="HazardCurvesLogLog">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55AD66A4-6C6C-40EB-B5E1-25D8F60F3127}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -31081,7 +31070,7 @@
         <xdr:cNvPr id="4" name="Chart 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -31119,7 +31108,7 @@
         <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -31157,7 +31146,7 @@
         <xdr:cNvPr id="6" name="Chart 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -31195,7 +31184,7 @@
         <xdr:cNvPr id="7" name="Chart 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000007000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -32390,7 +32379,7 @@
         <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -32428,7 +32417,7 @@
         <xdr:cNvPr id="7" name="Chart 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000007000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -32466,7 +32455,7 @@
         <xdr:cNvPr id="8" name="Chart 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000008000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -32504,7 +32493,7 @@
         <xdr:cNvPr id="9" name="Chart 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30AC2FE7-6C12-0A14-9E26-6D624A299C8B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000009000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -33110,7 +33099,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -36532,24 +36521,24 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="95" t="s">
+      <c r="A50" s="94" t="s">
         <v>39</v>
       </c>
-      <c r="B50" s="96" t="s">
+      <c r="B50" s="95" t="s">
         <v>44</v>
       </c>
-      <c r="C50" s="98" t="s">
+      <c r="C50" s="97" t="s">
         <v>36</v>
       </c>
-      <c r="D50" s="100" t="s">
+      <c r="D50" s="99" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="101"/>
+      <c r="E50" s="100"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="95"/>
-      <c r="B51" s="97"/>
-      <c r="C51" s="99"/>
+      <c r="A51" s="94"/>
+      <c r="B51" s="96"/>
+      <c r="C51" s="98"/>
       <c r="D51" s="4" t="s">
         <v>37</v>
       </c>
@@ -36781,7 +36770,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -37629,7 +37618,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -37757,7 +37746,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="102" t="s">
+      <c r="A4" s="101" t="s">
         <v>71</v>
       </c>
       <c r="B4" s="16" t="s">
@@ -37792,7 +37781,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="103"/>
+      <c r="A5" s="102"/>
       <c r="B5" s="20" t="s">
         <v>57</v>
       </c>
@@ -37825,7 +37814,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="104"/>
+      <c r="A6" s="103"/>
       <c r="B6" s="23" t="s">
         <v>58</v>
       </c>
@@ -37997,10 +37986,10 @@
       <c r="I13" s="38"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="105" t="s">
+      <c r="B14" s="104" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="106"/>
+      <c r="C14" s="105"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B15" s="30" t="s">
@@ -38280,7 +38269,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
@@ -38304,10 +38293,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="86" t="s">
+      <c r="B1" s="83" t="s">
         <v>62</v>
       </c>
       <c r="C1" s="50" t="s">
@@ -38393,7 +38382,7 @@
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A2" s="84">
+      <c r="A2" s="81">
         <f>$C$19*B2</f>
         <v>1.8500000000000001E-3</v>
       </c>
@@ -38483,7 +38472,7 @@
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A3" s="84">
+      <c r="A3" s="81">
         <f t="shared" ref="A3:A16" si="0">$C$19*B3</f>
         <v>3.3992640000000004E-3</v>
       </c>
@@ -38573,7 +38562,7 @@
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A4" s="84">
+      <c r="A4" s="81">
         <f t="shared" si="0"/>
         <v>6.2459145000000006E-3</v>
       </c>
@@ -38663,7 +38652,7 @@
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A5" s="84">
+      <c r="A5" s="81">
         <f t="shared" si="0"/>
         <v>1.1476456500000001E-2</v>
       </c>
@@ -38753,7 +38742,7 @@
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A6" s="84">
+      <c r="A6" s="81">
         <f t="shared" si="0"/>
         <v>2.1087225000000001E-2</v>
       </c>
@@ -38843,7 +38832,7 @@
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A7" s="84">
+      <c r="A7" s="81">
         <f t="shared" si="0"/>
         <v>3.8746585E-2</v>
       </c>
@@ -38933,7 +38922,7 @@
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A8" s="84">
+      <c r="A8" s="81">
         <f t="shared" si="0"/>
         <v>7.1194104999999994E-2</v>
       </c>
@@ -39023,7 +39012,7 @@
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A9" s="84">
+      <c r="A9" s="81">
         <f t="shared" si="0"/>
         <v>0.13081479500000001</v>
       </c>
@@ -39113,7 +39102,7 @@
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A10" s="84">
+      <c r="A10" s="81">
         <f t="shared" si="0"/>
         <v>0.24036310000000002</v>
       </c>
@@ -39203,7 +39192,7 @@
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A11" s="84">
+      <c r="A11" s="81">
         <f t="shared" si="0"/>
         <v>0.44165235000000003</v>
       </c>
@@ -39293,7 +39282,7 @@
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A12" s="84">
+      <c r="A12" s="81">
         <f t="shared" si="0"/>
         <v>0.81150805000000004</v>
       </c>
@@ -39383,7 +39372,7 @@
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A13" s="84">
+      <c r="A13" s="81">
         <f t="shared" si="0"/>
         <v>1.4910944500000001</v>
       </c>
@@ -39473,7 +39462,7 @@
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A14" s="84">
+      <c r="A14" s="81">
         <f t="shared" si="0"/>
         <v>2.7397944999999999</v>
       </c>
@@ -39563,7 +39552,7 @@
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A15" s="84">
+      <c r="A15" s="81">
         <f t="shared" si="0"/>
         <v>5.0341830000000005</v>
       </c>
@@ -39653,7 +39642,7 @@
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A16" s="84">
+      <c r="A16" s="81">
         <f t="shared" si="0"/>
         <v>9.25</v>
       </c>
@@ -39756,118 +39745,118 @@
       </c>
       <c r="C20" s="46"/>
     </row>
-    <row r="21" spans="1:29" s="88" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="87" t="s">
+    <row r="21" spans="1:29" s="85" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="B21" s="86" t="s">
+      <c r="B21" s="83" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="91" t="str">
+      <c r="C21" s="88" t="str">
         <f>"ln(λ_im("&amp;C1&amp;"))"</f>
         <v>ln(λ_im(T=0.01s))</v>
       </c>
-      <c r="D21" s="91" t="str">
+      <c r="D21" s="88" t="str">
         <f t="shared" ref="D21:AC21" si="1">"ln(λ_im("&amp;D1&amp;"))"</f>
         <v>ln(λ_im(T=0.015s))</v>
       </c>
-      <c r="E21" s="91" t="str">
+      <c r="E21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.02s))</v>
       </c>
-      <c r="F21" s="91" t="str">
+      <c r="F21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.03s))</v>
       </c>
-      <c r="G21" s="91" t="str">
+      <c r="G21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.04s))</v>
       </c>
-      <c r="H21" s="91" t="str">
+      <c r="H21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.05s))</v>
       </c>
-      <c r="I21" s="91" t="str">
+      <c r="I21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.06s))</v>
       </c>
-      <c r="J21" s="91" t="str">
+      <c r="J21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.075s))</v>
       </c>
-      <c r="K21" s="91" t="str">
+      <c r="K21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.09s))</v>
       </c>
-      <c r="L21" s="91" t="str">
+      <c r="L21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.1s))</v>
       </c>
-      <c r="M21" s="91" t="str">
+      <c r="M21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.15s))</v>
       </c>
-      <c r="N21" s="91" t="str">
+      <c r="N21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.2s))</v>
       </c>
-      <c r="O21" s="91" t="str">
+      <c r="O21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.3s))</v>
       </c>
-      <c r="P21" s="91" t="str">
+      <c r="P21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.4s))</v>
       </c>
-      <c r="Q21" s="91" t="str">
+      <c r="Q21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.5s))</v>
       </c>
-      <c r="R21" s="91" t="str">
+      <c r="R21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.6s))</v>
       </c>
-      <c r="S21" s="91" t="str">
+      <c r="S21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.7s))</v>
       </c>
-      <c r="T21" s="91" t="str">
+      <c r="T21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.75s))</v>
       </c>
-      <c r="U21" s="91" t="str">
+      <c r="U21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.8s))</v>
       </c>
-      <c r="V21" s="91" t="str">
+      <c r="V21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.9s))</v>
       </c>
-      <c r="W21" s="91" t="str">
+      <c r="W21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=1s))</v>
       </c>
-      <c r="X21" s="91" t="str">
+      <c r="X21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=1.2s))</v>
       </c>
-      <c r="Y21" s="91" t="str">
+      <c r="Y21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=1.5s))</v>
       </c>
-      <c r="Z21" s="91" t="str">
+      <c r="Z21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=2s))</v>
       </c>
-      <c r="AA21" s="91" t="str">
+      <c r="AA21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=2.5s))</v>
       </c>
-      <c r="AB21" s="91" t="str">
+      <c r="AB21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=3s))</v>
       </c>
-      <c r="AC21" s="91" t="str">
+      <c r="AC21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=5s))</v>
       </c>
@@ -39880,111 +39869,111 @@
       <c r="B22">
         <v>1E-3</v>
       </c>
-      <c r="C22" s="81">
+      <c r="C22" s="79">
         <f>LN(C2)</f>
         <v>0.14153248288198406</v>
       </c>
-      <c r="D22" s="81">
+      <c r="D22" s="79">
         <f t="shared" ref="D22:AC22" si="2">LN(D2)</f>
         <v>0.14794367328510374</v>
       </c>
-      <c r="E22" s="81">
+      <c r="E22" s="79">
         <f t="shared" si="2"/>
         <v>0.15392824152112117</v>
       </c>
-      <c r="F22" s="81">
+      <c r="F22" s="79">
         <f t="shared" si="2"/>
         <v>0.17141337226013387</v>
       </c>
-      <c r="G22" s="81">
+      <c r="G22" s="79">
         <f t="shared" si="2"/>
         <v>0.18829067688415135</v>
       </c>
-      <c r="H22" s="81">
+      <c r="H22" s="79">
         <f t="shared" si="2"/>
         <v>0.20965962905190849</v>
       </c>
-      <c r="I22" s="81">
+      <c r="I22" s="79">
         <f t="shared" si="2"/>
         <v>0.23683694926788029</v>
       </c>
-      <c r="J22" s="81">
+      <c r="J22" s="79">
         <f t="shared" si="2"/>
         <v>0.2736029585428863</v>
       </c>
-      <c r="K22" s="81">
+      <c r="K22" s="79">
         <f t="shared" si="2"/>
         <v>0.3016302633963916</v>
       </c>
-      <c r="L22" s="81">
+      <c r="L22" s="79">
         <f t="shared" si="2"/>
         <v>0.31755991606848488</v>
       </c>
-      <c r="M22" s="81">
+      <c r="M22" s="79">
         <f t="shared" si="2"/>
         <v>0.35094575114754295</v>
       </c>
-      <c r="N22" s="81">
+      <c r="N22" s="79">
         <f t="shared" si="2"/>
         <v>0.35757001895604612</v>
       </c>
-      <c r="O22" s="81">
+      <c r="O22" s="79">
         <f t="shared" si="2"/>
         <v>0.34446523702786386</v>
       </c>
-      <c r="P22" s="81">
+      <c r="P22" s="79">
         <f t="shared" si="2"/>
         <v>0.30654987124074184</v>
       </c>
-      <c r="Q22" s="81">
+      <c r="Q22" s="79">
         <f t="shared" si="2"/>
         <v>0.25020871342570428</v>
       </c>
-      <c r="R22" s="81">
+      <c r="R22" s="79">
         <f t="shared" si="2"/>
         <v>0.17649145317775991</v>
       </c>
-      <c r="S22" s="81">
+      <c r="S22" s="79">
         <f t="shared" si="2"/>
         <v>0.10287491179739859</v>
       </c>
-      <c r="T22" s="81">
+      <c r="T22" s="79">
         <f t="shared" si="2"/>
         <v>6.2787874884622508E-2</v>
       </c>
-      <c r="U22" s="81">
+      <c r="U22" s="79">
         <f t="shared" si="2"/>
         <v>2.8133460419483971E-2</v>
       </c>
-      <c r="V22" s="81">
+      <c r="V22" s="79">
         <f t="shared" si="2"/>
         <v>-4.6173640996181313E-2</v>
       </c>
-      <c r="W22" s="81">
+      <c r="W22" s="79">
         <f t="shared" si="2"/>
         <v>-0.13897069093715844</v>
       </c>
-      <c r="X22" s="81">
+      <c r="X22" s="79">
         <f t="shared" si="2"/>
         <v>-0.26623709141987334</v>
       </c>
-      <c r="Y22" s="81">
+      <c r="Y22" s="79">
         <f t="shared" si="2"/>
         <v>-0.49439446318786434</v>
       </c>
-      <c r="Z22" s="81">
+      <c r="Z22" s="79">
         <f t="shared" si="2"/>
         <v>-0.80723247833478662</v>
       </c>
-      <c r="AA22" s="81">
+      <c r="AA22" s="79">
         <f t="shared" si="2"/>
         <v>-1.0318443405444981</v>
       </c>
-      <c r="AB22" s="81">
+      <c r="AB22" s="79">
         <f t="shared" si="2"/>
         <v>-1.3037863414912909</v>
       </c>
-      <c r="AC22" s="81">
+      <c r="AC22" s="79">
         <f t="shared" si="2"/>
         <v>-1.734570175054909</v>
       </c>
@@ -39997,111 +39986,111 @@
       <c r="B23">
         <v>1.8374400000000001E-3</v>
       </c>
-      <c r="C23" s="81">
+      <c r="C23" s="79">
         <f t="shared" ref="C23:R36" si="4">LN(C3)</f>
         <v>-0.13276025077369941</v>
       </c>
-      <c r="D23" s="81">
+      <c r="D23" s="79">
         <f t="shared" si="4"/>
         <v>-0.12185393483829413</v>
       </c>
-      <c r="E23" s="81">
+      <c r="E23" s="79">
         <f t="shared" si="4"/>
         <v>-0.11153789618422746</v>
       </c>
-      <c r="F23" s="81">
+      <c r="F23" s="79">
         <f t="shared" si="4"/>
         <v>-8.4855759508759468E-2</v>
       </c>
-      <c r="G23" s="81">
+      <c r="G23" s="79">
         <f t="shared" si="4"/>
         <v>-5.9602112340752168E-2</v>
       </c>
-      <c r="H23" s="81">
+      <c r="H23" s="79">
         <f t="shared" si="4"/>
         <v>-3.3473932775435436E-2</v>
       </c>
-      <c r="I23" s="81">
+      <c r="I23" s="79">
         <f t="shared" si="4"/>
         <v>3.8665441745085504E-3</v>
       </c>
-      <c r="J23" s="81">
+      <c r="J23" s="79">
         <f t="shared" si="4"/>
         <v>4.8432695899548107E-2</v>
       </c>
-      <c r="K23" s="81">
+      <c r="K23" s="79">
         <f t="shared" si="4"/>
         <v>8.4963065949646754E-2</v>
       </c>
-      <c r="L23" s="81">
+      <c r="L23" s="79">
         <f t="shared" si="4"/>
         <v>0.10717021241990045</v>
       </c>
-      <c r="M23" s="81">
+      <c r="M23" s="79">
         <f t="shared" si="4"/>
         <v>0.14085668033083801</v>
       </c>
-      <c r="N23" s="81">
+      <c r="N23" s="79">
         <f t="shared" si="4"/>
         <v>0.14225841322312532</v>
       </c>
-      <c r="O23" s="81">
+      <c r="O23" s="79">
         <f t="shared" si="4"/>
         <v>0.11688093526837584</v>
       </c>
-      <c r="P23" s="81">
+      <c r="P23" s="79">
         <f t="shared" si="4"/>
         <v>6.2244392911600978E-2</v>
       </c>
-      <c r="Q23" s="81">
+      <c r="Q23" s="79">
         <f t="shared" si="4"/>
         <v>-1.7595247269446761E-2</v>
       </c>
-      <c r="R23" s="81">
+      <c r="R23" s="79">
         <f t="shared" si="4"/>
         <v>-0.11420176927791581</v>
       </c>
-      <c r="S23" s="81">
+      <c r="S23" s="79">
         <f t="shared" ref="S23:AC23" si="5">LN(S3)</f>
         <v>-0.20720005808756053</v>
       </c>
-      <c r="T23" s="81">
+      <c r="T23" s="79">
         <f t="shared" si="5"/>
         <v>-0.25631719438051709</v>
       </c>
-      <c r="U23" s="81">
+      <c r="U23" s="79">
         <f t="shared" si="5"/>
         <v>-0.30040493146758573</v>
       </c>
-      <c r="V23" s="81">
+      <c r="V23" s="79">
         <f t="shared" si="5"/>
         <v>-0.39400518410095331</v>
       </c>
-      <c r="W23" s="81">
+      <c r="W23" s="79">
         <f t="shared" si="5"/>
         <v>-0.50581924292992519</v>
       </c>
-      <c r="X23" s="81">
+      <c r="X23" s="79">
         <f t="shared" si="5"/>
         <v>-0.65396134204362344</v>
       </c>
-      <c r="Y23" s="81">
+      <c r="Y23" s="79">
         <f t="shared" si="5"/>
         <v>-0.91502069407619535</v>
       </c>
-      <c r="Z23" s="81">
+      <c r="Z23" s="79">
         <f t="shared" si="5"/>
         <v>-1.2645628543056087</v>
       </c>
-      <c r="AA23" s="81">
+      <c r="AA23" s="79">
         <f t="shared" si="5"/>
         <v>-1.5128495366885502</v>
       </c>
-      <c r="AB23" s="81">
+      <c r="AB23" s="79">
         <f t="shared" si="5"/>
         <v>-1.8145413121071432</v>
       </c>
-      <c r="AC23" s="81">
+      <c r="AC23" s="79">
         <f t="shared" si="5"/>
         <v>-2.2687526429924967</v>
       </c>
@@ -40114,111 +40103,111 @@
       <c r="B24">
         <v>3.37617E-3</v>
       </c>
-      <c r="C24" s="81">
+      <c r="C24" s="79">
         <f t="shared" si="4"/>
         <v>-0.49237956423522727</v>
       </c>
-      <c r="D24" s="81">
+      <c r="D24" s="79">
         <f t="shared" si="4"/>
         <v>-0.47629180155004419</v>
       </c>
-      <c r="E24" s="81">
+      <c r="E24" s="79">
         <f t="shared" si="4"/>
         <v>-0.46098273508407411</v>
       </c>
-      <c r="F24" s="81">
+      <c r="F24" s="79">
         <f t="shared" si="4"/>
         <v>-0.42373589806097933</v>
       </c>
-      <c r="G24" s="81">
+      <c r="G24" s="79">
         <f t="shared" si="4"/>
         <v>-0.38891762805619279</v>
       </c>
-      <c r="H24" s="81">
+      <c r="H24" s="79">
         <f t="shared" si="4"/>
         <v>-0.35554180358839255</v>
       </c>
-      <c r="I24" s="81">
+      <c r="I24" s="79">
         <f t="shared" si="4"/>
         <v>-0.30315863725568803</v>
       </c>
-      <c r="J24" s="81">
+      <c r="J24" s="79">
         <f t="shared" si="4"/>
         <v>-0.24578057010262366</v>
       </c>
-      <c r="K24" s="81">
+      <c r="K24" s="79">
         <f t="shared" si="4"/>
         <v>-0.20020659793706957</v>
       </c>
-      <c r="L24" s="81">
+      <c r="L24" s="79">
         <f t="shared" si="4"/>
         <v>-0.17216888884895029</v>
       </c>
-      <c r="M24" s="81">
+      <c r="M24" s="79">
         <f t="shared" si="4"/>
         <v>-0.1391994827344932</v>
       </c>
-      <c r="N24" s="81">
+      <c r="N24" s="79">
         <f t="shared" si="4"/>
         <v>-0.14491084745203006</v>
       </c>
-      <c r="O24" s="81">
+      <c r="O24" s="79">
         <f t="shared" si="4"/>
         <v>-0.19312042458214262</v>
       </c>
-      <c r="P24" s="81">
+      <c r="P24" s="79">
         <f t="shared" si="4"/>
         <v>-0.27317271578761382</v>
       </c>
-      <c r="Q24" s="81">
+      <c r="Q24" s="79">
         <f t="shared" si="4"/>
         <v>-0.37846501718989134</v>
       </c>
-      <c r="R24" s="81">
+      <c r="R24" s="79">
         <f t="shared" si="4"/>
         <v>-0.49456754498590205</v>
       </c>
-      <c r="S24" s="81">
+      <c r="S24" s="79">
         <f t="shared" ref="S24:AC24" si="6">LN(S4)</f>
         <v>-0.60673684933463767</v>
       </c>
-      <c r="T24" s="81">
+      <c r="T24" s="79">
         <f t="shared" si="6"/>
         <v>-0.66449864981020457</v>
       </c>
-      <c r="U24" s="81">
+      <c r="U24" s="79">
         <f t="shared" si="6"/>
         <v>-0.71583403751769803</v>
       </c>
-      <c r="V24" s="81">
+      <c r="V24" s="79">
         <f t="shared" si="6"/>
         <v>-0.82366507541902512</v>
       </c>
-      <c r="W24" s="81">
+      <c r="W24" s="79">
         <f t="shared" si="6"/>
         <v>-0.94998195423525267</v>
       </c>
-      <c r="X24" s="81">
+      <c r="X24" s="79">
         <f t="shared" si="6"/>
         <v>-1.1156792358438654</v>
       </c>
-      <c r="Y24" s="81">
+      <c r="Y24" s="79">
         <f t="shared" si="6"/>
         <v>-1.4062672199974438</v>
       </c>
-      <c r="Z24" s="81">
+      <c r="Z24" s="79">
         <f t="shared" si="6"/>
         <v>-1.7896876542296991</v>
       </c>
-      <c r="AA24" s="81">
+      <c r="AA24" s="79">
         <f t="shared" si="6"/>
         <v>-2.0610589875437606</v>
       </c>
-      <c r="AB24" s="81">
+      <c r="AB24" s="79">
         <f t="shared" si="6"/>
         <v>-2.3919212372167307</v>
       </c>
-      <c r="AC24" s="81">
+      <c r="AC24" s="79">
         <f t="shared" si="6"/>
         <v>-2.8697712186722732</v>
       </c>
@@ -40231,111 +40220,111 @@
       <c r="B25">
         <v>6.2034899999999999E-3</v>
       </c>
-      <c r="C25" s="81">
+      <c r="C25" s="79">
         <f t="shared" si="4"/>
         <v>-0.93797294069738213</v>
       </c>
-      <c r="D25" s="81">
+      <c r="D25" s="79">
         <f t="shared" si="4"/>
         <v>-0.91614658624613521</v>
       </c>
-      <c r="E25" s="81">
+      <c r="E25" s="79">
         <f t="shared" si="4"/>
         <v>-0.89532610251296907</v>
       </c>
-      <c r="F25" s="81">
+      <c r="F25" s="79">
         <f t="shared" si="4"/>
         <v>-0.84688917028238286</v>
       </c>
-      <c r="G25" s="81">
+      <c r="G25" s="79">
         <f t="shared" si="4"/>
         <v>-0.80181011762694521</v>
       </c>
-      <c r="H25" s="81">
+      <c r="H25" s="79">
         <f t="shared" si="4"/>
         <v>-0.75967824762412717</v>
       </c>
-      <c r="I25" s="81">
+      <c r="I25" s="79">
         <f t="shared" si="4"/>
         <v>-0.6896208337218297</v>
       </c>
-      <c r="J25" s="81">
+      <c r="J25" s="79">
         <f t="shared" si="4"/>
         <v>-0.61562816427229772</v>
       </c>
-      <c r="K25" s="81">
+      <c r="K25" s="79">
         <f t="shared" si="4"/>
         <v>-0.55955960111343184</v>
       </c>
-      <c r="L25" s="81">
+      <c r="L25" s="79">
         <f t="shared" si="4"/>
         <v>-0.5253633412105897</v>
       </c>
-      <c r="M25" s="81">
+      <c r="M25" s="79">
         <f t="shared" si="4"/>
         <v>-0.4960645699945358</v>
       </c>
-      <c r="N25" s="81">
+      <c r="N25" s="79">
         <f t="shared" si="4"/>
         <v>-0.51398851206784635</v>
       </c>
-      <c r="O25" s="81">
+      <c r="O25" s="79">
         <f t="shared" si="4"/>
         <v>-0.59537915386473073</v>
       </c>
-      <c r="P25" s="81">
+      <c r="P25" s="79">
         <f t="shared" si="4"/>
         <v>-0.70196589955888933</v>
       </c>
-      <c r="Q25" s="81">
+      <c r="Q25" s="79">
         <f t="shared" si="4"/>
         <v>-0.82865870068644543</v>
       </c>
-      <c r="R25" s="81">
+      <c r="R25" s="79">
         <f t="shared" si="4"/>
         <v>-0.9608088891996398</v>
       </c>
-      <c r="S25" s="81">
+      <c r="S25" s="79">
         <f t="shared" ref="S25:AC25" si="7">LN(S5)</f>
         <v>-1.0893366697878217</v>
       </c>
-      <c r="T25" s="81">
+      <c r="T25" s="79">
         <f t="shared" si="7"/>
         <v>-1.1551210579416165</v>
       </c>
-      <c r="U25" s="81">
+      <c r="U25" s="79">
         <f t="shared" si="7"/>
         <v>-1.2122504096846043</v>
       </c>
-      <c r="V25" s="81">
+      <c r="V25" s="79">
         <f t="shared" si="7"/>
         <v>-1.3321545763308318</v>
       </c>
-      <c r="W25" s="81">
+      <c r="W25" s="79">
         <f t="shared" si="7"/>
         <v>-1.4719717514974355</v>
       </c>
-      <c r="X25" s="81">
+      <c r="X25" s="79">
         <f t="shared" si="7"/>
         <v>-1.6528901611253972</v>
       </c>
-      <c r="Y25" s="81">
+      <c r="Y25" s="79">
         <f t="shared" si="7"/>
         <v>-1.969103779835609</v>
       </c>
-      <c r="Z25" s="81">
+      <c r="Z25" s="79">
         <f t="shared" si="7"/>
         <v>-2.3865696344375484</v>
       </c>
-      <c r="AA25" s="81">
+      <c r="AA25" s="79">
         <f t="shared" si="7"/>
         <v>-2.6795873124021736</v>
       </c>
-      <c r="AB25" s="81">
+      <c r="AB25" s="79">
         <f t="shared" si="7"/>
         <v>-3.0377294766947935</v>
       </c>
-      <c r="AC25" s="81">
+      <c r="AC25" s="79">
         <f t="shared" si="7"/>
         <v>-3.5401342650116372</v>
       </c>
@@ -40348,111 +40337,111 @@
       <c r="B26">
         <v>1.1398500000000001E-2</v>
       </c>
-      <c r="C26" s="81">
+      <c r="C26" s="79">
         <f t="shared" si="4"/>
         <v>-1.4667820205889468</v>
       </c>
-      <c r="D26" s="81">
+      <c r="D26" s="79">
         <f t="shared" si="4"/>
         <v>-1.438548671500685</v>
       </c>
-      <c r="E26" s="81">
+      <c r="E26" s="79">
         <f t="shared" si="4"/>
         <v>-1.411586792154178</v>
       </c>
-      <c r="F26" s="81">
+      <c r="F26" s="79">
         <f t="shared" si="4"/>
         <v>-1.3513113828796186</v>
       </c>
-      <c r="G26" s="81">
+      <c r="G26" s="79">
         <f t="shared" si="4"/>
         <v>-1.2952808475599742</v>
       </c>
-      <c r="H26" s="81">
+      <c r="H26" s="79">
         <f t="shared" si="4"/>
         <v>-1.2433952288326247</v>
       </c>
-      <c r="I26" s="81">
+      <c r="I26" s="79">
         <f t="shared" si="4"/>
         <v>-1.1555017093593829</v>
       </c>
-      <c r="J26" s="81">
+      <c r="J26" s="79">
         <f t="shared" si="4"/>
         <v>-1.0626661339758681</v>
       </c>
-      <c r="K26" s="81">
+      <c r="K26" s="79">
         <f t="shared" si="4"/>
         <v>-0.99555745878983792</v>
       </c>
-      <c r="L26" s="81">
+      <c r="L26" s="79">
         <f t="shared" si="4"/>
         <v>-0.95497217662677136</v>
       </c>
-      <c r="M26" s="81">
+      <c r="M26" s="79">
         <f t="shared" si="4"/>
         <v>-0.93224572067400613</v>
       </c>
-      <c r="N26" s="81">
+      <c r="N26" s="79">
         <f t="shared" si="4"/>
         <v>-0.96640801515654762</v>
       </c>
-      <c r="O26" s="81">
+      <c r="O26" s="79">
         <f t="shared" si="4"/>
         <v>-1.0865396817723727</v>
       </c>
-      <c r="P26" s="81">
+      <c r="P26" s="79">
         <f t="shared" si="4"/>
         <v>-1.2178517118578431</v>
       </c>
-      <c r="Q26" s="81">
+      <c r="Q26" s="79">
         <f t="shared" si="4"/>
         <v>-1.3614410571308295</v>
       </c>
-      <c r="R26" s="81">
+      <c r="R26" s="79">
         <f t="shared" si="4"/>
         <v>-1.5069346710170375</v>
       </c>
-      <c r="S26" s="81">
+      <c r="S26" s="79">
         <f t="shared" ref="S26:AC26" si="8">LN(S6)</f>
         <v>-1.6502212685029134</v>
       </c>
-      <c r="T26" s="81">
+      <c r="T26" s="79">
         <f t="shared" si="8"/>
         <v>-1.7238306670901491</v>
       </c>
-      <c r="U26" s="81">
+      <c r="U26" s="79">
         <f t="shared" si="8"/>
         <v>-1.7860114109861758</v>
       </c>
-      <c r="V26" s="81">
+      <c r="V26" s="79">
         <f t="shared" si="8"/>
         <v>-1.9176263252986652</v>
       </c>
-      <c r="W26" s="81">
+      <c r="W26" s="79">
         <f t="shared" si="8"/>
         <v>-2.0711805023894136</v>
       </c>
-      <c r="X26" s="81">
+      <c r="X26" s="79">
         <f t="shared" si="8"/>
         <v>-2.2663076113185792</v>
       </c>
-      <c r="Y26" s="81">
+      <c r="Y26" s="79">
         <f t="shared" si="8"/>
         <v>-2.6055856167904947</v>
       </c>
-      <c r="Z26" s="81">
+      <c r="Z26" s="79">
         <f t="shared" si="8"/>
         <v>-3.0560321516263835</v>
       </c>
-      <c r="AA26" s="81">
+      <c r="AA26" s="79">
         <f t="shared" si="8"/>
         <v>-3.3715668472118741</v>
       </c>
-      <c r="AB26" s="81">
+      <c r="AB26" s="79">
         <f t="shared" si="8"/>
         <v>-3.7544235559167145</v>
       </c>
-      <c r="AC26" s="81">
+      <c r="AC26" s="79">
         <f t="shared" si="8"/>
         <v>-4.2843780642300029</v>
       </c>
@@ -40465,111 +40454,111 @@
       <c r="B27">
         <v>2.09441E-2</v>
       </c>
-      <c r="C27" s="81">
+      <c r="C27" s="79">
         <f t="shared" si="4"/>
         <v>-2.0752129475884846</v>
       </c>
-      <c r="D27" s="81">
+      <c r="D27" s="79">
         <f t="shared" si="4"/>
         <v>-2.0403318070608445</v>
       </c>
-      <c r="E27" s="81">
+      <c r="E27" s="79">
         <f t="shared" si="4"/>
         <v>-2.006950001420587</v>
       </c>
-      <c r="F27" s="81">
+      <c r="F27" s="79">
         <f t="shared" si="4"/>
         <v>-1.9348420034974174</v>
       </c>
-      <c r="G27" s="81">
+      <c r="G27" s="79">
         <f t="shared" si="4"/>
         <v>-1.867640066074006</v>
       </c>
-      <c r="H27" s="81">
+      <c r="H27" s="79">
         <f t="shared" si="4"/>
         <v>-1.8054863375104266</v>
       </c>
-      <c r="I27" s="81">
+      <c r="I27" s="79">
         <f t="shared" si="4"/>
         <v>-1.7011611987101372</v>
       </c>
-      <c r="J27" s="81">
+      <c r="J27" s="79">
         <f t="shared" si="4"/>
         <v>-1.5893126496400714</v>
       </c>
-      <c r="K27" s="81">
+      <c r="K27" s="79">
         <f t="shared" si="4"/>
         <v>-1.5121515067187759</v>
       </c>
-      <c r="L27" s="81">
+      <c r="L27" s="79">
         <f t="shared" si="4"/>
         <v>-1.4653683934502859</v>
       </c>
-      <c r="M27" s="81">
+      <c r="M27" s="79">
         <f t="shared" si="4"/>
         <v>-1.4511093248765323</v>
       </c>
-      <c r="N27" s="81">
+      <c r="N27" s="79">
         <f t="shared" si="4"/>
         <v>-1.5022677898157233</v>
       </c>
-      <c r="O27" s="81">
+      <c r="O27" s="79">
         <f t="shared" si="4"/>
         <v>-1.6622218895108978</v>
       </c>
-      <c r="P27" s="81">
+      <c r="P27" s="79">
         <f t="shared" si="4"/>
         <v>-1.8136556726816397</v>
       </c>
-      <c r="Q27" s="81">
+      <c r="Q27" s="79">
         <f t="shared" si="4"/>
         <v>-1.9696352120274254</v>
       </c>
-      <c r="R27" s="81">
+      <c r="R27" s="79">
         <f t="shared" si="4"/>
         <v>-2.1273048283414098</v>
       </c>
-      <c r="S27" s="81">
+      <c r="S27" s="79">
         <f t="shared" ref="S27:AC27" si="9">LN(S7)</f>
         <v>-2.2851293333877845</v>
       </c>
-      <c r="T27" s="81">
+      <c r="T27" s="79">
         <f t="shared" si="9"/>
         <v>-2.3666606868595164</v>
       </c>
-      <c r="U27" s="81">
+      <c r="U27" s="79">
         <f t="shared" si="9"/>
         <v>-2.4338387058918443</v>
       </c>
-      <c r="V27" s="81">
+      <c r="V27" s="79">
         <f t="shared" si="9"/>
         <v>-2.5773462747028324</v>
       </c>
-      <c r="W27" s="81">
+      <c r="W27" s="79">
         <f t="shared" si="9"/>
         <v>-2.7446549617591991</v>
       </c>
-      <c r="X27" s="81">
+      <c r="X27" s="79">
         <f t="shared" si="9"/>
         <v>-2.9529966697495689</v>
       </c>
-      <c r="Y27" s="81">
+      <c r="Y27" s="79">
         <f t="shared" si="9"/>
         <v>-3.3144696720795706</v>
       </c>
-      <c r="Z27" s="81">
+      <c r="Z27" s="79">
         <f t="shared" si="9"/>
         <v>-3.7952158454538027</v>
       </c>
-      <c r="AA27" s="81">
+      <c r="AA27" s="79">
         <f t="shared" si="9"/>
         <v>-4.1340088497450358</v>
       </c>
-      <c r="AB27" s="81">
+      <c r="AB27" s="79">
         <f t="shared" si="9"/>
         <v>-4.5381165875491094</v>
       </c>
-      <c r="AC27" s="81">
+      <c r="AC27" s="79">
         <f t="shared" si="9"/>
         <v>-5.1089448686280896</v>
       </c>
@@ -40582,111 +40571,111 @@
       <c r="B28">
         <v>3.8483299999999998E-2</v>
       </c>
-      <c r="C28" s="81">
+      <c r="C28" s="79">
         <f t="shared" si="4"/>
         <v>-2.757494999192017</v>
       </c>
-      <c r="D28" s="81">
+      <c r="D28" s="79">
         <f t="shared" si="4"/>
         <v>-2.7156432360956684</v>
       </c>
-      <c r="E28" s="81">
+      <c r="E28" s="79">
         <f t="shared" si="4"/>
         <v>-2.6756410398697188</v>
       </c>
-      <c r="F28" s="81">
+      <c r="F28" s="79">
         <f t="shared" si="4"/>
         <v>-2.5921399513570509</v>
       </c>
-      <c r="G28" s="81">
+      <c r="G28" s="79">
         <f t="shared" si="4"/>
         <v>-2.5144301504992339</v>
       </c>
-      <c r="H28" s="81">
+      <c r="H28" s="79">
         <f t="shared" si="4"/>
         <v>-2.4427031603989611</v>
       </c>
-      <c r="I28" s="81">
+      <c r="I28" s="79">
         <f t="shared" si="4"/>
         <v>-2.3264309656353994</v>
       </c>
-      <c r="J28" s="81">
+      <c r="J28" s="79">
         <f t="shared" si="4"/>
         <v>-2.1977535657413738</v>
       </c>
-      <c r="K28" s="81">
+      <c r="K28" s="79">
         <f t="shared" si="4"/>
         <v>-2.113320477030626</v>
       </c>
-      <c r="L28" s="81">
+      <c r="L28" s="79">
         <f t="shared" si="4"/>
         <v>-2.0614228939032957</v>
       </c>
-      <c r="M28" s="81">
+      <c r="M28" s="79">
         <f t="shared" si="4"/>
         <v>-2.0557104135529731</v>
       </c>
-      <c r="N28" s="81">
+      <c r="N28" s="79">
         <f t="shared" si="4"/>
         <v>-2.1207459740188526</v>
       </c>
-      <c r="O28" s="81">
+      <c r="O28" s="79">
         <f t="shared" si="4"/>
         <v>-2.3153497931174063</v>
       </c>
-      <c r="P28" s="81">
+      <c r="P28" s="79">
         <f t="shared" si="4"/>
         <v>-2.4817156922693124</v>
       </c>
-      <c r="Q28" s="81">
+      <c r="Q28" s="79">
         <f t="shared" si="4"/>
         <v>-2.6478441996645663</v>
       </c>
-      <c r="R28" s="81">
+      <c r="R28" s="79">
         <f t="shared" si="4"/>
         <v>-2.817750921886228</v>
       </c>
-      <c r="S28" s="81">
+      <c r="S28" s="79">
         <f t="shared" ref="S28:AC28" si="10">LN(S8)</f>
         <v>-2.9902235093570297</v>
       </c>
-      <c r="T28" s="81">
+      <c r="T28" s="79">
         <f t="shared" si="10"/>
         <v>-3.0793041597763553</v>
       </c>
-      <c r="U28" s="81">
+      <c r="U28" s="79">
         <f t="shared" si="10"/>
         <v>-3.1513725702942619</v>
       </c>
-      <c r="V28" s="81">
+      <c r="V28" s="79">
         <f t="shared" si="10"/>
         <v>-3.3063762619943371</v>
       </c>
-      <c r="W28" s="81">
+      <c r="W28" s="79">
         <f t="shared" si="10"/>
         <v>-3.4868909803866117</v>
       </c>
-      <c r="X28" s="81">
+      <c r="X28" s="79">
         <f t="shared" si="10"/>
         <v>-3.7078924192386431</v>
       </c>
-      <c r="Y28" s="81">
+      <c r="Y28" s="79">
         <f t="shared" si="10"/>
         <v>-4.0904942879690136</v>
       </c>
-      <c r="Z28" s="81">
+      <c r="Z28" s="79">
         <f t="shared" si="10"/>
         <v>-4.6030720428233787</v>
       </c>
-      <c r="AA28" s="81">
+      <c r="AA28" s="79">
         <f t="shared" si="10"/>
         <v>-4.9652616067097934</v>
       </c>
-      <c r="AB28" s="81">
+      <c r="AB28" s="79">
         <f t="shared" si="10"/>
         <v>-5.3866806686673829</v>
       </c>
-      <c r="AC28" s="81">
+      <c r="AC28" s="79">
         <f t="shared" si="10"/>
         <v>-6.0434821066109814</v>
       </c>
@@ -40699,111 +40688,111 @@
       <c r="B29">
         <v>7.0710700000000001E-2</v>
       </c>
-      <c r="C29" s="81">
+      <c r="C29" s="79">
         <f t="shared" si="4"/>
         <v>-3.5219082952496907</v>
       </c>
-      <c r="D29" s="81">
+      <c r="D29" s="79">
         <f t="shared" si="4"/>
         <v>-3.4716883620209673</v>
       </c>
-      <c r="E29" s="81">
+      <c r="E29" s="79">
         <f t="shared" si="4"/>
         <v>-3.4238012113781835</v>
       </c>
-      <c r="F29" s="81">
+      <c r="F29" s="79">
         <f t="shared" si="4"/>
         <v>-3.3266538752078834</v>
       </c>
-      <c r="G29" s="81">
+      <c r="G29" s="79">
         <f t="shared" si="4"/>
         <v>-3.2368673191425694</v>
       </c>
-      <c r="H29" s="81">
+      <c r="H29" s="79">
         <f t="shared" si="4"/>
         <v>-3.1545921331676872</v>
       </c>
-      <c r="I29" s="81">
+      <c r="I29" s="79">
         <f t="shared" si="4"/>
         <v>-3.0285815186168037</v>
       </c>
-      <c r="J29" s="81">
+      <c r="J29" s="79">
         <f t="shared" si="4"/>
         <v>-2.8857837617599182</v>
       </c>
-      <c r="K29" s="81">
+      <c r="K29" s="79">
         <f t="shared" si="4"/>
         <v>-2.7985471999538203</v>
       </c>
-      <c r="L29" s="81">
+      <c r="L29" s="79">
         <f t="shared" si="4"/>
         <v>-2.7434951098186251</v>
       </c>
-      <c r="M29" s="81">
+      <c r="M29" s="79">
         <f t="shared" si="4"/>
         <v>-2.7431715429910906</v>
       </c>
-      <c r="N29" s="81">
+      <c r="N29" s="79">
         <f t="shared" si="4"/>
         <v>-2.815949588742797</v>
       </c>
-      <c r="O29" s="81">
+      <c r="O29" s="79">
         <f t="shared" si="4"/>
         <v>-3.0402083726014308</v>
       </c>
-      <c r="P29" s="81">
+      <c r="P29" s="79">
         <f t="shared" si="4"/>
         <v>-3.2191042403846812</v>
       </c>
-      <c r="Q29" s="81">
+      <c r="Q29" s="79">
         <f t="shared" si="4"/>
         <v>-3.395439350743672</v>
       </c>
-      <c r="R29" s="81">
+      <c r="R29" s="79">
         <f t="shared" si="4"/>
         <v>-3.5788180810396262</v>
       </c>
-      <c r="S29" s="81">
+      <c r="S29" s="79">
         <f t="shared" ref="S29:AC29" si="11">LN(S9)</f>
         <v>-3.7658006648753575</v>
       </c>
-      <c r="T29" s="81">
+      <c r="T29" s="79">
         <f t="shared" si="11"/>
         <v>-3.8614781024070237</v>
       </c>
-      <c r="U29" s="81">
+      <c r="U29" s="79">
         <f t="shared" si="11"/>
         <v>-3.9382052254194995</v>
       </c>
-      <c r="V29" s="81">
+      <c r="V29" s="79">
         <f t="shared" si="11"/>
         <v>-4.1039981059910371</v>
       </c>
-      <c r="W29" s="81">
+      <c r="W29" s="79">
         <f t="shared" si="11"/>
         <v>-4.2966434554375894</v>
       </c>
-      <c r="X29" s="81">
+      <c r="X29" s="79">
         <f t="shared" si="11"/>
         <v>-4.5314638605058626</v>
       </c>
-      <c r="Y29" s="81">
+      <c r="Y29" s="79">
         <f t="shared" si="11"/>
         <v>-4.9363249770015623</v>
       </c>
-      <c r="Z29" s="81">
+      <c r="Z29" s="79">
         <f t="shared" si="11"/>
         <v>-5.4878956580616371</v>
       </c>
-      <c r="AA29" s="81">
+      <c r="AA29" s="79">
         <f t="shared" si="11"/>
         <v>-5.8796046193858649</v>
       </c>
-      <c r="AB29" s="81">
+      <c r="AB29" s="79">
         <f t="shared" si="11"/>
         <v>-6.3199747112851021</v>
       </c>
-      <c r="AC29" s="81">
+      <c r="AC29" s="79">
         <f t="shared" si="11"/>
         <v>-7.1379279696699749</v>
       </c>
@@ -40816,111 +40805,111 @@
       <c r="B30">
         <v>0.12992600000000001</v>
       </c>
-      <c r="C30" s="81">
+      <c r="C30" s="79">
         <f t="shared" si="4"/>
         <v>-4.3956284172629472</v>
       </c>
-      <c r="D30" s="81">
+      <c r="D30" s="79">
         <f t="shared" si="4"/>
         <v>-4.3349768563042836</v>
       </c>
-      <c r="E30" s="81">
+      <c r="E30" s="79">
         <f t="shared" si="4"/>
         <v>-4.2771936549430487</v>
       </c>
-      <c r="F30" s="81">
+      <c r="F30" s="79">
         <f t="shared" si="4"/>
         <v>-4.1619307938293977</v>
       </c>
-      <c r="G30" s="81">
+      <c r="G30" s="79">
         <f t="shared" si="4"/>
         <v>-4.0561417657244885</v>
       </c>
-      <c r="H30" s="81">
+      <c r="H30" s="79">
         <f t="shared" si="4"/>
         <v>-3.9599111939788822</v>
       </c>
-      <c r="I30" s="81">
+      <c r="I30" s="79">
         <f t="shared" si="4"/>
         <v>-3.8201161282935256</v>
       </c>
-      <c r="J30" s="81">
+      <c r="J30" s="79">
         <f t="shared" si="4"/>
         <v>-3.6606116888194538</v>
       </c>
-      <c r="K30" s="81">
+      <c r="K30" s="79">
         <f t="shared" si="4"/>
         <v>-3.5715062282625856</v>
       </c>
-      <c r="L30" s="81">
+      <c r="L30" s="79">
         <f t="shared" si="4"/>
         <v>-3.5137583545278646</v>
       </c>
-      <c r="M30" s="81">
+      <c r="M30" s="79">
         <f t="shared" si="4"/>
         <v>-3.5146775403493593</v>
       </c>
-      <c r="N30" s="81">
+      <c r="N30" s="79">
         <f t="shared" si="4"/>
         <v>-3.5907497000984625</v>
       </c>
-      <c r="O30" s="81">
+      <c r="O30" s="79">
         <f t="shared" si="4"/>
         <v>-3.8418477945117435</v>
       </c>
-      <c r="P30" s="81">
+      <c r="P30" s="79">
         <f t="shared" si="4"/>
         <v>-4.0322229780724461</v>
       </c>
-      <c r="Q30" s="81">
+      <c r="Q30" s="79">
         <f t="shared" si="4"/>
         <v>-4.2202519457598804</v>
       </c>
-      <c r="R30" s="81">
+      <c r="R30" s="79">
         <f t="shared" si="4"/>
         <v>-4.4188142700466537</v>
       </c>
-      <c r="S30" s="81">
+      <c r="S30" s="79">
         <f t="shared" ref="S30:AC30" si="12">LN(S10)</f>
         <v>-4.6190594943747065</v>
       </c>
-      <c r="T30" s="81">
+      <c r="T30" s="79">
         <f t="shared" si="12"/>
         <v>-4.7195795599030212</v>
       </c>
-      <c r="U30" s="81">
+      <c r="U30" s="79">
         <f t="shared" si="12"/>
         <v>-4.8005129197670895</v>
       </c>
-      <c r="V30" s="81">
+      <c r="V30" s="79">
         <f t="shared" si="12"/>
         <v>-4.9765590754274704</v>
       </c>
-      <c r="W30" s="81">
+      <c r="W30" s="79">
         <f t="shared" si="12"/>
         <v>-5.1798055717891316</v>
       </c>
-      <c r="X30" s="81">
+      <c r="X30" s="79">
         <f t="shared" si="12"/>
         <v>-5.4302742778884241</v>
       </c>
-      <c r="Y30" s="81">
+      <c r="Y30" s="79">
         <f t="shared" si="12"/>
         <v>-5.8622797441763277</v>
       </c>
-      <c r="Z30" s="81">
+      <c r="Z30" s="79">
         <f t="shared" si="12"/>
         <v>-6.4657988962812212</v>
       </c>
-      <c r="AA30" s="81">
+      <c r="AA30" s="79">
         <f t="shared" si="12"/>
         <v>-6.9009401575210907</v>
       </c>
-      <c r="AB30" s="81">
+      <c r="AB30" s="79">
         <f t="shared" si="12"/>
         <v>-7.3768224512162446</v>
       </c>
-      <c r="AC30" s="81">
+      <c r="AC30" s="79">
         <f t="shared" si="12"/>
         <v>-8.4716211825968557</v>
       </c>
@@ -40933,111 +40922,111 @@
       <c r="B31">
         <v>0.238731</v>
       </c>
-      <c r="C31" s="81">
+      <c r="C31" s="79">
         <f t="shared" si="4"/>
         <v>-5.4210716780558315</v>
       </c>
-      <c r="D31" s="81">
+      <c r="D31" s="79">
         <f t="shared" si="4"/>
         <v>-5.348008292554999</v>
       </c>
-      <c r="E31" s="81">
+      <c r="E31" s="79">
         <f t="shared" si="4"/>
         <v>-5.2782126259161091</v>
       </c>
-      <c r="F31" s="81">
+      <c r="F31" s="79">
         <f t="shared" si="4"/>
         <v>-5.1393135185582448</v>
       </c>
-      <c r="G31" s="81">
+      <c r="G31" s="79">
         <f t="shared" si="4"/>
         <v>-5.0122302493433315</v>
       </c>
-      <c r="H31" s="81">
+      <c r="H31" s="79">
         <f t="shared" si="4"/>
         <v>-4.8968593823136475</v>
       </c>
-      <c r="I31" s="81">
+      <c r="I31" s="79">
         <f t="shared" si="4"/>
         <v>-4.7338031391224353</v>
       </c>
-      <c r="J31" s="81">
+      <c r="J31" s="79">
         <f t="shared" si="4"/>
         <v>-4.5496671564163433</v>
       </c>
-      <c r="K31" s="81">
+      <c r="K31" s="79">
         <f t="shared" si="4"/>
         <v>-4.4536492246227857</v>
       </c>
-      <c r="L31" s="81">
+      <c r="L31" s="79">
         <f t="shared" si="4"/>
         <v>-4.3903500392423966</v>
       </c>
-      <c r="M31" s="81">
+      <c r="M31" s="79">
         <f t="shared" si="4"/>
         <v>-4.3860955090982952</v>
       </c>
-      <c r="N31" s="81">
+      <c r="N31" s="79">
         <f t="shared" si="4"/>
         <v>-4.4627805609704776</v>
       </c>
-      <c r="O31" s="81">
+      <c r="O31" s="79">
         <f t="shared" si="4"/>
         <v>-4.7379620152446353</v>
       </c>
-      <c r="P31" s="81">
+      <c r="P31" s="79">
         <f t="shared" si="4"/>
         <v>-4.9381220098089011</v>
       </c>
-      <c r="Q31" s="81">
+      <c r="Q31" s="79">
         <f t="shared" si="4"/>
         <v>-5.1394290861704111</v>
       </c>
-      <c r="R31" s="81">
+      <c r="R31" s="79">
         <f t="shared" si="4"/>
         <v>-5.3555445803624862</v>
       </c>
-      <c r="S31" s="81">
+      <c r="S31" s="79">
         <f t="shared" ref="S31:AC31" si="13">LN(S11)</f>
         <v>-5.5669079887240729</v>
       </c>
-      <c r="T31" s="81">
+      <c r="T31" s="79">
         <f t="shared" si="13"/>
         <v>-5.6698343051473286</v>
       </c>
-      <c r="U31" s="81">
+      <c r="U31" s="79">
         <f t="shared" si="13"/>
         <v>-5.7541629843282198</v>
       </c>
-      <c r="V31" s="81">
+      <c r="V31" s="79">
         <f t="shared" si="13"/>
         <v>-5.9392050795093638</v>
       </c>
-      <c r="W31" s="81">
+      <c r="W31" s="79">
         <f t="shared" si="13"/>
         <v>-6.1517278675214468</v>
       </c>
-      <c r="X31" s="81">
+      <c r="X31" s="79">
         <f t="shared" si="13"/>
         <v>-6.4189611907620439</v>
       </c>
-      <c r="Y31" s="81">
+      <c r="Y31" s="79">
         <f t="shared" si="13"/>
         <v>-6.8905256767471963</v>
       </c>
-      <c r="Z31" s="81">
+      <c r="Z31" s="79">
         <f t="shared" si="13"/>
         <v>-7.5920775565174319</v>
       </c>
-      <c r="AA31" s="81">
+      <c r="AA31" s="79">
         <f t="shared" si="13"/>
         <v>-8.115538058523553</v>
       </c>
-      <c r="AB31" s="81">
+      <c r="AB31" s="79">
         <f t="shared" si="13"/>
         <v>-8.6842141340460515</v>
       </c>
-      <c r="AC31" s="81">
+      <c r="AC31" s="79">
         <f t="shared" si="13"/>
         <v>-10.27909009813078</v>
       </c>
@@ -41050,111 +41039,111 @@
       <c r="B32">
         <v>0.43865300000000002</v>
       </c>
-      <c r="C32" s="81">
+      <c r="C32" s="79">
         <f t="shared" si="4"/>
         <v>-6.6678644795798654</v>
       </c>
-      <c r="D32" s="81">
+      <c r="D32" s="79">
         <f t="shared" si="4"/>
         <v>-6.580212461010416</v>
       </c>
-      <c r="E32" s="81">
+      <c r="E32" s="79">
         <f t="shared" si="4"/>
         <v>-6.4958729776292445</v>
       </c>
-      <c r="F32" s="81">
+      <c r="F32" s="79">
         <f t="shared" si="4"/>
         <v>-6.3252420941677476</v>
       </c>
-      <c r="G32" s="81">
+      <c r="G32" s="79">
         <f t="shared" si="4"/>
         <v>-6.1691518703912713</v>
       </c>
-      <c r="H32" s="81">
+      <c r="H32" s="79">
         <f t="shared" si="4"/>
         <v>-6.0269900549560909</v>
       </c>
-      <c r="I32" s="81">
+      <c r="I32" s="79">
         <f t="shared" si="4"/>
         <v>-5.8223024196480857</v>
       </c>
-      <c r="J32" s="81">
+      <c r="J32" s="79">
         <f t="shared" si="4"/>
         <v>-5.5992009830874077</v>
       </c>
-      <c r="K32" s="81">
+      <c r="K32" s="79">
         <f t="shared" si="4"/>
         <v>-5.4836955943514534</v>
       </c>
-      <c r="L32" s="81">
+      <c r="L32" s="79">
         <f t="shared" si="4"/>
         <v>-5.4072127913947003</v>
       </c>
-      <c r="M32" s="81">
+      <c r="M32" s="79">
         <f t="shared" si="4"/>
         <v>-5.3862021293115161</v>
       </c>
-      <c r="N32" s="81">
+      <c r="N32" s="79">
         <f t="shared" si="4"/>
         <v>-5.4628107231229421</v>
       </c>
-      <c r="O32" s="81">
+      <c r="O32" s="79">
         <f t="shared" si="4"/>
         <v>-5.7601129565272196</v>
       </c>
-      <c r="P32" s="81">
+      <c r="P32" s="79">
         <f t="shared" si="4"/>
         <v>-5.9685536850065262</v>
       </c>
-      <c r="Q32" s="81">
+      <c r="Q32" s="79">
         <f t="shared" si="4"/>
         <v>-6.1849335267237304</v>
       </c>
-      <c r="R32" s="81">
+      <c r="R32" s="79">
         <f t="shared" si="4"/>
         <v>-6.423601876300995</v>
       </c>
-      <c r="S32" s="81">
+      <c r="S32" s="79">
         <f t="shared" ref="S32:AC32" si="14">LN(S12)</f>
         <v>-6.6432693461419712</v>
       </c>
-      <c r="T32" s="81">
+      <c r="T32" s="79">
         <f t="shared" si="14"/>
         <v>-6.7453290376117874</v>
       </c>
-      <c r="U32" s="81">
+      <c r="U32" s="79">
         <f t="shared" si="14"/>
         <v>-6.8315866617908778</v>
       </c>
-      <c r="V32" s="81">
+      <c r="V32" s="79">
         <f t="shared" si="14"/>
         <v>-7.0253597615322221</v>
       </c>
-      <c r="W32" s="81">
+      <c r="W32" s="79">
         <f t="shared" si="14"/>
         <v>-7.251020530322144</v>
       </c>
-      <c r="X32" s="81">
+      <c r="X32" s="79">
         <f t="shared" si="14"/>
         <v>-7.5437686550417267</v>
       </c>
-      <c r="Y32" s="81">
+      <c r="Y32" s="79">
         <f t="shared" si="14"/>
         <v>-8.1065105365275389</v>
       </c>
-      <c r="Z32" s="81">
+      <c r="Z32" s="79">
         <f t="shared" si="14"/>
         <v>-9.0210796247120815</v>
       </c>
-      <c r="AA32" s="81">
+      <c r="AA32" s="79">
         <f t="shared" si="14"/>
         <v>-9.7388311159933636</v>
       </c>
-      <c r="AB32" s="81">
+      <c r="AB32" s="79">
         <f t="shared" si="14"/>
         <v>-10.518190444118162</v>
       </c>
-      <c r="AC32" s="81">
+      <c r="AC32" s="79">
         <f t="shared" si="14"/>
         <v>-12.478747264008026</v>
       </c>
@@ -41167,111 +41156,111 @@
       <c r="B33">
         <v>0.80599699999999996</v>
       </c>
-      <c r="C33" s="81">
+      <c r="C33" s="79">
         <f t="shared" si="4"/>
         <v>-8.2149322946834236</v>
       </c>
-      <c r="D33" s="81">
+      <c r="D33" s="79">
         <f t="shared" si="4"/>
         <v>-8.1148016604242912</v>
       </c>
-      <c r="E33" s="81">
+      <c r="E33" s="79">
         <f t="shared" si="4"/>
         <v>-8.0168048378778654</v>
       </c>
-      <c r="F33" s="81">
+      <c r="F33" s="79">
         <f t="shared" si="4"/>
         <v>-7.8082316843158583</v>
       </c>
-      <c r="G33" s="81">
+      <c r="G33" s="79">
         <f t="shared" si="4"/>
         <v>-7.6161100410509448</v>
       </c>
-      <c r="H33" s="81">
+      <c r="H33" s="79">
         <f t="shared" si="4"/>
         <v>-7.4395193543391827</v>
       </c>
-      <c r="I33" s="81">
+      <c r="I33" s="79">
         <f t="shared" si="4"/>
         <v>-7.1729316262772995</v>
       </c>
-      <c r="J33" s="81">
+      <c r="J33" s="79">
         <f t="shared" si="4"/>
         <v>-6.8827074962315624</v>
       </c>
-      <c r="K33" s="81">
+      <c r="K33" s="79">
         <f t="shared" si="4"/>
         <v>-6.7251067702361604</v>
       </c>
-      <c r="L33" s="81">
+      <c r="L33" s="79">
         <f t="shared" si="4"/>
         <v>-6.6218382191170777</v>
       </c>
-      <c r="M33" s="81">
+      <c r="M33" s="79">
         <f t="shared" si="4"/>
         <v>-6.5635960235655473</v>
       </c>
-      <c r="N33" s="81">
+      <c r="N33" s="79">
         <f t="shared" si="4"/>
         <v>-6.6458128005848671</v>
       </c>
-      <c r="O33" s="81">
+      <c r="O33" s="79">
         <f t="shared" si="4"/>
         <v>-6.9673362098233529</v>
       </c>
-      <c r="P33" s="81">
+      <c r="P33" s="79">
         <f t="shared" si="4"/>
         <v>-7.1784805904807749</v>
       </c>
-      <c r="Q33" s="81">
+      <c r="Q33" s="79">
         <f t="shared" si="4"/>
         <v>-7.4158301860269349</v>
       </c>
-      <c r="R33" s="81">
+      <c r="R33" s="79">
         <f t="shared" si="4"/>
         <v>-7.6852853717812906</v>
       </c>
-      <c r="S33" s="81">
+      <c r="S33" s="79">
         <f t="shared" ref="S33:AC33" si="15">LN(S13)</f>
         <v>-7.9097914797406057</v>
       </c>
-      <c r="T33" s="81">
+      <c r="T33" s="79">
         <f t="shared" si="15"/>
         <v>-8.0120259499645918</v>
       </c>
-      <c r="U33" s="81">
+      <c r="U33" s="79">
         <f t="shared" si="15"/>
         <v>-8.1036445132265484</v>
       </c>
-      <c r="V33" s="81">
+      <c r="V33" s="79">
         <f t="shared" si="15"/>
         <v>-8.3171091025007193</v>
       </c>
-      <c r="W33" s="81">
+      <c r="W33" s="79">
         <f t="shared" si="15"/>
         <v>-8.5713359997584124</v>
       </c>
-      <c r="X33" s="81">
+      <c r="X33" s="79">
         <f t="shared" si="15"/>
         <v>-8.926439593833452</v>
       </c>
-      <c r="Y33" s="81">
+      <c r="Y33" s="79">
         <f t="shared" si="15"/>
         <v>-9.681285942496956</v>
       </c>
-      <c r="Z33" s="81">
+      <c r="Z33" s="79">
         <f t="shared" si="15"/>
         <v>-10.840187405218693</v>
       </c>
-      <c r="AA33" s="81">
+      <c r="AA33" s="79">
         <f t="shared" si="15"/>
         <v>-11.814411255615953</v>
       </c>
-      <c r="AB33" s="81">
+      <c r="AB33" s="79">
         <f t="shared" si="15"/>
         <v>-12.826106725014634</v>
       </c>
-      <c r="AC33" s="81">
+      <c r="AC33" s="79">
         <f t="shared" si="15"/>
         <v>-14.706470815510418</v>
       </c>
@@ -41284,111 +41273,111 @@
       <c r="B34">
         <v>1.4809699999999999</v>
       </c>
-      <c r="C34" s="81">
+      <c r="C34" s="79">
         <f t="shared" si="4"/>
         <v>-10.075691951339543</v>
       </c>
-      <c r="D34" s="81">
+      <c r="D34" s="79">
         <f t="shared" si="4"/>
         <v>-9.9678750255425097</v>
       </c>
-      <c r="E34" s="81">
+      <c r="E34" s="79">
         <f t="shared" si="4"/>
         <v>-9.8599628025993358</v>
       </c>
-      <c r="F34" s="81">
+      <c r="F34" s="79">
         <f t="shared" si="4"/>
         <v>-9.6118029655372617</v>
       </c>
-      <c r="G34" s="81">
+      <c r="G34" s="79">
         <f t="shared" si="4"/>
         <v>-9.3817719914328634</v>
       </c>
-      <c r="H34" s="81">
+      <c r="H34" s="79">
         <f t="shared" si="4"/>
         <v>-9.168732115341518</v>
       </c>
-      <c r="I34" s="81">
+      <c r="I34" s="79">
         <f t="shared" si="4"/>
         <v>-8.8452209228167149</v>
       </c>
-      <c r="J34" s="81">
+      <c r="J34" s="79">
         <f t="shared" si="4"/>
         <v>-8.4480315073146226</v>
       </c>
-      <c r="K34" s="81">
+      <c r="K34" s="79">
         <f t="shared" si="4"/>
         <v>-8.223125068162874</v>
       </c>
-      <c r="L34" s="81">
+      <c r="L34" s="79">
         <f t="shared" si="4"/>
         <v>-8.076540457727555</v>
       </c>
-      <c r="M34" s="81">
+      <c r="M34" s="79">
         <f t="shared" si="4"/>
         <v>-7.9565201705012463</v>
       </c>
-      <c r="N34" s="81">
+      <c r="N34" s="79">
         <f t="shared" si="4"/>
         <v>-8.0652350219095013</v>
       </c>
-      <c r="O34" s="81">
+      <c r="O34" s="79">
         <f t="shared" si="4"/>
         <v>-8.4150993858970136</v>
       </c>
-      <c r="P34" s="81">
+      <c r="P34" s="79">
         <f t="shared" si="4"/>
         <v>-8.5985901463868935</v>
       </c>
-      <c r="Q34" s="81">
+      <c r="Q34" s="79">
         <f t="shared" si="4"/>
         <v>-8.8712707272030276</v>
       </c>
-      <c r="R34" s="81">
+      <c r="R34" s="79">
         <f t="shared" si="4"/>
         <v>-9.1711298221309043</v>
       </c>
-      <c r="S34" s="81">
+      <c r="S34" s="79">
         <f t="shared" ref="S34:AC34" si="16">LN(S14)</f>
         <v>-9.3966949254961882</v>
       </c>
-      <c r="T34" s="81">
+      <c r="T34" s="79">
         <f t="shared" si="16"/>
         <v>-9.5086877098652245</v>
       </c>
-      <c r="U34" s="81">
+      <c r="U34" s="79">
         <f t="shared" si="16"/>
         <v>-9.6171713930081371</v>
       </c>
-      <c r="V34" s="81">
+      <c r="V34" s="79">
         <f t="shared" si="16"/>
         <v>-9.8754656533446727</v>
       </c>
-      <c r="W34" s="81">
+      <c r="W34" s="79">
         <f t="shared" si="16"/>
         <v>-10.170858576770165</v>
       </c>
-      <c r="X34" s="81">
+      <c r="X34" s="79">
         <f t="shared" si="16"/>
         <v>-10.641491785184501</v>
       </c>
-      <c r="Y34" s="81">
+      <c r="Y34" s="79">
         <f t="shared" si="16"/>
         <v>-11.639871907499554</v>
       </c>
-      <c r="Z34" s="81">
+      <c r="Z34" s="79">
         <f t="shared" si="16"/>
         <v>-13.026570403411105</v>
       </c>
-      <c r="AA34" s="81">
+      <c r="AA34" s="79">
         <f t="shared" si="16"/>
         <v>-14.237694593573512</v>
       </c>
-      <c r="AB34" s="81">
+      <c r="AB34" s="79">
         <f t="shared" si="16"/>
         <v>-15.457335944622089</v>
       </c>
-      <c r="AC34" s="81">
+      <c r="AC34" s="79">
         <f t="shared" si="16"/>
         <v>-17.063716078228335</v>
       </c>
@@ -41401,111 +41390,111 @@
       <c r="B35">
         <v>2.7211799999999999</v>
       </c>
-      <c r="C35" s="81">
+      <c r="C35" s="79">
         <f t="shared" si="4"/>
         <v>-12.318722768157366</v>
       </c>
-      <c r="D35" s="81">
+      <c r="D35" s="79">
         <f t="shared" si="4"/>
         <v>-12.202851846104247</v>
       </c>
-      <c r="E35" s="81">
+      <c r="E35" s="79">
         <f t="shared" si="4"/>
         <v>-12.083628458888162</v>
       </c>
-      <c r="F35" s="81">
+      <c r="F35" s="79">
         <f t="shared" si="4"/>
         <v>-11.786341109282578</v>
       </c>
-      <c r="G35" s="81">
+      <c r="G35" s="79">
         <f t="shared" si="4"/>
         <v>-11.509212753137078</v>
       </c>
-      <c r="H35" s="81">
+      <c r="H35" s="79">
         <f t="shared" si="4"/>
         <v>-11.25110221502112</v>
       </c>
-      <c r="I35" s="81">
+      <c r="I35" s="79">
         <f t="shared" si="4"/>
         <v>-10.842836466285892</v>
       </c>
-      <c r="J35" s="81">
+      <c r="J35" s="79">
         <f t="shared" si="4"/>
         <v>-10.313328570742764</v>
       </c>
-      <c r="K35" s="81">
+      <c r="K35" s="79">
         <f t="shared" si="4"/>
         <v>-9.9958846663524028</v>
       </c>
-      <c r="L35" s="81">
+      <c r="L35" s="79">
         <f t="shared" si="4"/>
         <v>-9.7866039505105693</v>
       </c>
-      <c r="M35" s="81">
+      <c r="M35" s="79">
         <f t="shared" si="4"/>
         <v>-9.5827757781568845</v>
       </c>
-      <c r="N35" s="81">
+      <c r="N35" s="79">
         <f t="shared" si="4"/>
         <v>-9.7369119222290514</v>
       </c>
-      <c r="O35" s="81">
+      <c r="O35" s="79">
         <f t="shared" si="4"/>
         <v>-10.114482511487122</v>
       </c>
-      <c r="P35" s="81">
+      <c r="P35" s="79">
         <f t="shared" si="4"/>
         <v>-10.250701517634557</v>
       </c>
-      <c r="Q35" s="81">
+      <c r="Q35" s="79">
         <f t="shared" si="4"/>
         <v>-10.575838548562608</v>
       </c>
-      <c r="R35" s="81">
+      <c r="R35" s="79">
         <f t="shared" si="4"/>
         <v>-10.9142571996573</v>
       </c>
-      <c r="S35" s="81">
+      <c r="S35" s="79">
         <f t="shared" ref="S35:AC35" si="17">LN(S15)</f>
         <v>-11.165037996542484</v>
       </c>
-      <c r="T35" s="81">
+      <c r="T35" s="79">
         <f t="shared" si="17"/>
         <v>-11.297941141285376</v>
       </c>
-      <c r="U35" s="81">
+      <c r="U35" s="79">
         <f t="shared" si="17"/>
         <v>-11.43202353042521</v>
       </c>
-      <c r="V35" s="81">
+      <c r="V35" s="79">
         <f t="shared" si="17"/>
         <v>-11.747595413276755</v>
       </c>
-      <c r="W35" s="81">
+      <c r="W35" s="79">
         <f t="shared" si="17"/>
         <v>-12.102716717394197</v>
       </c>
-      <c r="X35" s="81">
+      <c r="X35" s="79">
         <f t="shared" si="17"/>
         <v>-12.720269899576465</v>
       </c>
-      <c r="Y35" s="81">
+      <c r="Y35" s="79">
         <f t="shared" si="17"/>
         <v>-13.998208863683175</v>
       </c>
-      <c r="Z35" s="81">
+      <c r="Z35" s="79">
         <f t="shared" si="17"/>
         <v>-15.693752504768586</v>
       </c>
-      <c r="AA35" s="81">
+      <c r="AA35" s="79">
         <f t="shared" si="17"/>
         <v>-17.123158688412911</v>
       </c>
-      <c r="AB35" s="81">
+      <c r="AB35" s="79">
         <f t="shared" si="17"/>
         <v>-18.505451514189133</v>
       </c>
-      <c r="AC35" s="81">
+      <c r="AC35" s="79">
         <f t="shared" si="17"/>
         <v>-19.602262137587722</v>
       </c>
@@ -41518,292 +41507,292 @@
       <c r="B36">
         <v>5</v>
       </c>
-      <c r="C36" s="81">
+      <c r="C36" s="79">
         <f t="shared" si="4"/>
         <v>-15.007855668134352</v>
       </c>
-      <c r="D36" s="81">
+      <c r="D36" s="79">
         <f t="shared" si="4"/>
         <v>-14.880399109821674</v>
       </c>
-      <c r="E36" s="81">
+      <c r="E36" s="79">
         <f t="shared" si="4"/>
         <v>-14.74569591622949</v>
       </c>
-      <c r="F36" s="81">
+      <c r="F36" s="79">
         <f t="shared" si="4"/>
         <v>-14.390796815792442</v>
       </c>
-      <c r="G36" s="81">
+      <c r="G36" s="79">
         <f t="shared" si="4"/>
         <v>-14.058460852267594</v>
       </c>
-      <c r="H36" s="81">
+      <c r="H36" s="79">
         <f t="shared" si="4"/>
         <v>-13.747507719279874</v>
       </c>
-      <c r="I36" s="81">
+      <c r="I36" s="79">
         <f t="shared" si="4"/>
         <v>-13.241988634806207</v>
       </c>
-      <c r="J36" s="81">
+      <c r="J36" s="79">
         <f t="shared" si="4"/>
         <v>-12.567007504103742</v>
       </c>
-      <c r="K36" s="81">
+      <c r="K36" s="79">
         <f t="shared" si="4"/>
         <v>-12.136173925646682</v>
       </c>
-      <c r="L36" s="81">
+      <c r="L36" s="79">
         <f t="shared" si="4"/>
         <v>-11.845552613416812</v>
       </c>
-      <c r="M36" s="81">
+      <c r="M36" s="79">
         <f t="shared" si="4"/>
         <v>-11.54295152541458</v>
       </c>
-      <c r="N36" s="81">
+      <c r="N36" s="79">
         <f t="shared" si="4"/>
         <v>-11.751418959733629</v>
       </c>
-      <c r="O36" s="81">
+      <c r="O36" s="79">
         <f t="shared" si="4"/>
         <v>-12.165307487247368</v>
       </c>
-      <c r="P36" s="81">
+      <c r="P36" s="79">
         <f t="shared" si="4"/>
         <v>-12.251113112957</v>
       </c>
-      <c r="Q36" s="81">
+      <c r="Q36" s="79">
         <f t="shared" si="4"/>
         <v>-12.646024090743081</v>
       </c>
-      <c r="R36" s="81">
+      <c r="R36" s="79">
         <f t="shared" si="4"/>
         <v>-13.046175431266562</v>
       </c>
-      <c r="S36" s="81">
+      <c r="S36" s="79">
         <f t="shared" ref="S36:AC36" si="18">LN(S16)</f>
         <v>-13.352171020410557</v>
       </c>
-      <c r="T36" s="81">
+      <c r="T36" s="79">
         <f t="shared" si="18"/>
         <v>-13.517145049393916</v>
       </c>
-      <c r="U36" s="81">
+      <c r="U36" s="79">
         <f t="shared" si="18"/>
         <v>-13.684564960730295</v>
       </c>
-      <c r="V36" s="81">
+      <c r="V36" s="79">
         <f t="shared" si="18"/>
         <v>-14.068530419288823</v>
       </c>
-      <c r="W36" s="81">
+      <c r="W36" s="79">
         <f t="shared" si="18"/>
         <v>-14.502667383334495</v>
       </c>
-      <c r="X36" s="81">
+      <c r="X36" s="79">
         <f t="shared" si="18"/>
         <v>-15.285583827391743</v>
       </c>
-      <c r="Y36" s="81">
+      <c r="Y36" s="79">
         <f t="shared" si="18"/>
         <v>-16.86816240759936</v>
       </c>
-      <c r="Z36" s="81">
+      <c r="Z36" s="79">
         <f t="shared" si="18"/>
         <v>-18.884127808188023</v>
       </c>
-      <c r="AA36" s="81">
+      <c r="AA36" s="79">
         <f t="shared" si="18"/>
         <v>-20.438269835864521</v>
       </c>
-      <c r="AB36" s="81">
+      <c r="AB36" s="79">
         <f t="shared" si="18"/>
         <v>-21.835825467022293</v>
       </c>
-      <c r="AC36" s="81">
+      <c r="AC36" s="79">
         <f t="shared" si="18"/>
         <v>-22.369047717115379</v>
       </c>
     </row>
     <row r="37" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="C37" s="81"/>
-      <c r="D37" s="81"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="81"/>
-      <c r="G37" s="81"/>
-      <c r="H37" s="81"/>
-      <c r="I37" s="81"/>
-      <c r="J37" s="81"/>
-      <c r="K37" s="81"/>
-      <c r="L37" s="81"/>
-      <c r="M37" s="81"/>
-      <c r="N37" s="81"/>
-      <c r="O37" s="81"/>
-      <c r="P37" s="81"/>
-      <c r="Q37" s="81"/>
-      <c r="R37" s="81"/>
-      <c r="S37" s="81"/>
-      <c r="T37" s="81"/>
-      <c r="U37" s="81"/>
-      <c r="V37" s="81"/>
-      <c r="W37" s="81"/>
-      <c r="X37" s="81"/>
-      <c r="Y37" s="81"/>
-      <c r="Z37" s="81"/>
-      <c r="AA37" s="81"/>
-      <c r="AB37" s="81"/>
-      <c r="AC37" s="81"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="79"/>
+      <c r="E37" s="79"/>
+      <c r="F37" s="79"/>
+      <c r="G37" s="79"/>
+      <c r="H37" s="79"/>
+      <c r="I37" s="79"/>
+      <c r="J37" s="79"/>
+      <c r="K37" s="79"/>
+      <c r="L37" s="79"/>
+      <c r="M37" s="79"/>
+      <c r="N37" s="79"/>
+      <c r="O37" s="79"/>
+      <c r="P37" s="79"/>
+      <c r="Q37" s="79"/>
+      <c r="R37" s="79"/>
+      <c r="S37" s="79"/>
+      <c r="T37" s="79"/>
+      <c r="U37" s="79"/>
+      <c r="V37" s="79"/>
+      <c r="W37" s="79"/>
+      <c r="X37" s="79"/>
+      <c r="Y37" s="79"/>
+      <c r="Z37" s="79"/>
+      <c r="AA37" s="79"/>
+      <c r="AB37" s="79"/>
+      <c r="AC37" s="79"/>
     </row>
     <row r="38" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="C38" s="81"/>
-      <c r="D38" s="81"/>
-      <c r="E38" s="81"/>
-      <c r="F38" s="81"/>
-      <c r="G38" s="81"/>
-      <c r="H38" s="81"/>
-      <c r="I38" s="81"/>
-      <c r="J38" s="81"/>
-      <c r="K38" s="81"/>
-      <c r="L38" s="81"/>
-      <c r="M38" s="81"/>
-      <c r="N38" s="81"/>
-      <c r="O38" s="81"/>
-      <c r="P38" s="81"/>
-      <c r="Q38" s="81"/>
-      <c r="R38" s="81"/>
-      <c r="S38" s="81"/>
-      <c r="T38" s="81"/>
-      <c r="U38" s="81"/>
-      <c r="V38" s="81"/>
-      <c r="W38" s="81"/>
-      <c r="X38" s="81"/>
-      <c r="Y38" s="81">
+      <c r="C38" s="79"/>
+      <c r="D38" s="79"/>
+      <c r="E38" s="79"/>
+      <c r="F38" s="79"/>
+      <c r="G38" s="79"/>
+      <c r="H38" s="79"/>
+      <c r="I38" s="79"/>
+      <c r="J38" s="79"/>
+      <c r="K38" s="79"/>
+      <c r="L38" s="79"/>
+      <c r="M38" s="79"/>
+      <c r="N38" s="79"/>
+      <c r="O38" s="79"/>
+      <c r="P38" s="79"/>
+      <c r="Q38" s="79"/>
+      <c r="R38" s="79"/>
+      <c r="S38" s="79"/>
+      <c r="T38" s="79"/>
+      <c r="U38" s="79"/>
+      <c r="V38" s="79"/>
+      <c r="W38" s="79"/>
+      <c r="X38" s="79"/>
+      <c r="Y38" s="79">
         <v>1.5</v>
       </c>
-      <c r="Z38" s="81">
+      <c r="Z38" s="79">
         <v>2</v>
       </c>
-      <c r="AA38" s="81"/>
-      <c r="AB38" s="81"/>
-      <c r="AC38" s="81"/>
-      <c r="AF38" s="81">
+      <c r="AA38" s="79"/>
+      <c r="AB38" s="79"/>
+      <c r="AC38" s="79"/>
+      <c r="AF38" s="79">
         <v>1.84</v>
       </c>
     </row>
     <row r="39" spans="1:32" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="93" t="str">
+      <c r="C39" s="90" t="str">
         <f>"Sa("&amp;C1&amp;")"</f>
         <v>Sa(T=0.01s)</v>
       </c>
-      <c r="D39" s="93" t="str">
+      <c r="D39" s="90" t="str">
         <f t="shared" ref="D39:AC39" si="19">"Sa("&amp;D1&amp;")"</f>
         <v>Sa(T=0.015s)</v>
       </c>
-      <c r="E39" s="93" t="str">
+      <c r="E39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.02s)</v>
       </c>
-      <c r="F39" s="93" t="str">
+      <c r="F39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.03s)</v>
       </c>
-      <c r="G39" s="93" t="str">
+      <c r="G39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.04s)</v>
       </c>
-      <c r="H39" s="93" t="str">
+      <c r="H39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.05s)</v>
       </c>
-      <c r="I39" s="93" t="str">
+      <c r="I39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.06s)</v>
       </c>
-      <c r="J39" s="93" t="str">
+      <c r="J39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.075s)</v>
       </c>
-      <c r="K39" s="93" t="str">
+      <c r="K39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.09s)</v>
       </c>
-      <c r="L39" s="93" t="str">
+      <c r="L39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.1s)</v>
       </c>
-      <c r="M39" s="93" t="str">
+      <c r="M39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.15s)</v>
       </c>
-      <c r="N39" s="93" t="str">
+      <c r="N39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.2s)</v>
       </c>
-      <c r="O39" s="93" t="str">
+      <c r="O39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.3s)</v>
       </c>
-      <c r="P39" s="93" t="str">
+      <c r="P39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.4s)</v>
       </c>
-      <c r="Q39" s="93" t="str">
+      <c r="Q39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.5s)</v>
       </c>
-      <c r="R39" s="93" t="str">
+      <c r="R39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.6s)</v>
       </c>
-      <c r="S39" s="93" t="str">
+      <c r="S39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.7s)</v>
       </c>
-      <c r="T39" s="93" t="str">
+      <c r="T39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.75s)</v>
       </c>
-      <c r="U39" s="93" t="str">
+      <c r="U39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.8s)</v>
       </c>
-      <c r="V39" s="93" t="str">
+      <c r="V39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.9s)</v>
       </c>
-      <c r="W39" s="93" t="str">
+      <c r="W39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=1s)</v>
       </c>
-      <c r="X39" s="93" t="str">
+      <c r="X39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=1.2s)</v>
       </c>
-      <c r="Y39" s="93" t="str">
+      <c r="Y39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=1.5s)</v>
       </c>
-      <c r="Z39" s="93" t="str">
+      <c r="Z39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=2s)</v>
       </c>
-      <c r="AA39" s="93" t="str">
+      <c r="AA39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=2.5s)</v>
       </c>
-      <c r="AB39" s="93" t="str">
+      <c r="AB39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=3s)</v>
       </c>
-      <c r="AC39" s="93" t="str">
+      <c r="AC39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=5s)</v>
       </c>
     </row>
     <row r="40" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="92" t="s">
+      <c r="A40" s="89" t="s">
         <v>106</v>
       </c>
       <c r="C40">
@@ -41916,7 +41905,7 @@
       </c>
     </row>
     <row r="41" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="92" t="s">
+      <c r="A41" s="89" t="s">
         <v>105</v>
       </c>
       <c r="C41">
@@ -42033,43 +42022,43 @@
       </c>
     </row>
     <row r="43" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="83" t="s">
+      <c r="A43" s="80" t="s">
         <v>103</v>
       </c>
-      <c r="C43" s="85">
+      <c r="C43" s="82">
         <f ca="1">(E53-C40)/C40</f>
         <v>-0.21186959173753381</v>
       </c>
-      <c r="W43" s="85">
+      <c r="W43" s="82">
         <f ca="1">(F53-W40)/W40</f>
         <v>0.12487578274156814</v>
       </c>
-      <c r="Y43" s="85">
+      <c r="Y43" s="82">
         <f ca="1">(G53-Y40)/Y40</f>
         <v>0.16053579176207786</v>
       </c>
-      <c r="Z43" s="85">
+      <c r="Z43" s="82">
         <f ca="1">(H53-Z40)/Z40</f>
         <v>0.25544497928350646</v>
       </c>
     </row>
     <row r="44" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="83" t="s">
+      <c r="A44" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="C44" s="85">
+      <c r="C44" s="82">
         <f ca="1">(E56-C41)/C41</f>
         <v>-0.41111685662093045</v>
       </c>
-      <c r="W44" s="85">
+      <c r="W44" s="82">
         <f ca="1">(F56-W41)/W41</f>
         <v>-0.28696676621404749</v>
       </c>
-      <c r="Y44" s="85">
+      <c r="Y44" s="82">
         <f ca="1">(G56-Y41)/Y41</f>
         <v>-0.28676023868652284</v>
       </c>
-      <c r="Z44" s="85">
+      <c r="Z44" s="82">
         <f ca="1">(H56-Z41)/Z41</f>
         <v>-0.22746236568769571</v>
       </c>
@@ -42080,36 +42069,36 @@
       </c>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B49" s="76" t="s">
+      <c r="B49" s="75" t="s">
         <v>39</v>
       </c>
-      <c r="C49" s="76" t="s">
+      <c r="C49" s="75" t="s">
         <v>44</v>
       </c>
-      <c r="D49" s="76" t="s">
+      <c r="D49" s="75" t="s">
         <v>36</v>
       </c>
-      <c r="E49" s="107" t="s">
+      <c r="E49" s="92" t="s">
         <v>41</v>
       </c>
-      <c r="F49" s="108"/>
-      <c r="G49" s="108"/>
-      <c r="H49" s="108"/>
+      <c r="F49" s="93"/>
+      <c r="G49" s="93"/>
+      <c r="H49" s="93"/>
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B50" s="76"/>
-      <c r="C50" s="76"/>
-      <c r="D50" s="76"/>
-      <c r="E50" s="76" t="s">
+      <c r="B50" s="75"/>
+      <c r="C50" s="75"/>
+      <c r="D50" s="75"/>
+      <c r="E50" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="F50" s="76" t="s">
+      <c r="F50" s="75" t="s">
         <v>40</v>
       </c>
-      <c r="G50" s="76" t="s">
+      <c r="G50" s="75" t="s">
         <v>92</v>
       </c>
-      <c r="H50" s="76" t="s">
+      <c r="H50" s="75" t="s">
         <v>93</v>
       </c>
     </row>
@@ -42118,6 +42107,7 @@
         <v>175</v>
       </c>
       <c r="C51" s="3">
+        <f t="shared" ref="C51:C58" si="22">1/B51</f>
         <v>5.7142857142857143E-3</v>
       </c>
       <c r="D51" s="5">
@@ -42145,25 +42135,26 @@
         <v>275</v>
       </c>
       <c r="C52" s="3">
+        <f t="shared" si="22"/>
         <v>3.6363636363636364E-3</v>
       </c>
       <c r="D52" s="5">
         <v>0.45</v>
       </c>
       <c r="E52" s="5">
-        <f t="shared" ref="E52:E58" si="22">(D52*$E$66)</f>
+        <f t="shared" ref="E52:E58" si="23">(D52*$E$66)</f>
         <v>0.45</v>
       </c>
       <c r="F52" s="5">
-        <f t="shared" ref="F52:F58" si="23">(D52*$F$66)</f>
+        <f t="shared" ref="F52:F58" si="24">(D52*$F$66)</f>
         <v>0.45</v>
       </c>
       <c r="G52" s="5">
-        <f t="shared" ref="G52:G58" si="24">(D52*$G$66)</f>
+        <f t="shared" ref="G52:G58" si="25">(D52*$G$66)</f>
         <v>0.3</v>
       </c>
       <c r="H52" s="5">
-        <f t="shared" ref="H52:H58" si="25">(D52*$H$66)</f>
+        <f t="shared" ref="H52:H58" si="26">(D52*$H$66)</f>
         <v>0.22500000000000001</v>
       </c>
     </row>
@@ -42172,25 +42163,26 @@
         <v>475</v>
       </c>
       <c r="C53" s="48">
+        <f t="shared" si="22"/>
         <v>2.1052631578947368E-3</v>
       </c>
       <c r="D53" s="49">
         <v>0.5</v>
       </c>
       <c r="E53" s="49">
-        <f t="shared" si="22"/>
-        <v>0.5</v>
-      </c>
-      <c r="F53" s="49">
         <f t="shared" si="23"/>
         <v>0.5</v>
       </c>
+      <c r="F53" s="49">
+        <f t="shared" si="24"/>
+        <v>0.5</v>
+      </c>
       <c r="G53" s="49">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.33333333333333331</v>
       </c>
       <c r="H53" s="49">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.25</v>
       </c>
     </row>
@@ -42199,25 +42191,26 @@
         <v>975</v>
       </c>
       <c r="C54" s="3">
+        <f t="shared" si="22"/>
         <v>1.0256410256410256E-3</v>
       </c>
       <c r="D54" s="5">
         <v>0.6</v>
       </c>
       <c r="E54" s="5">
-        <f t="shared" si="22"/>
-        <v>0.6</v>
-      </c>
-      <c r="F54" s="5">
         <f t="shared" si="23"/>
         <v>0.6</v>
       </c>
+      <c r="F54" s="5">
+        <f t="shared" si="24"/>
+        <v>0.6</v>
+      </c>
       <c r="G54" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.39999999999999997</v>
       </c>
       <c r="H54" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.3</v>
       </c>
     </row>
@@ -42226,25 +42219,26 @@
         <v>1275</v>
       </c>
       <c r="C55" s="3">
+        <f t="shared" si="22"/>
         <v>7.8431372549019605E-4</v>
       </c>
       <c r="D55" s="5">
         <v>0.625</v>
       </c>
       <c r="E55" s="5">
-        <f t="shared" si="22"/>
-        <v>0.625</v>
-      </c>
-      <c r="F55" s="5">
         <f t="shared" si="23"/>
         <v>0.625</v>
       </c>
+      <c r="F55" s="5">
+        <f t="shared" si="24"/>
+        <v>0.625</v>
+      </c>
       <c r="G55" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.41666666666666663</v>
       </c>
       <c r="H55" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.3125</v>
       </c>
     </row>
@@ -42253,25 +42247,26 @@
         <v>2475</v>
       </c>
       <c r="C56" s="48">
+        <f t="shared" si="22"/>
         <v>4.0404040404040404E-4</v>
       </c>
       <c r="D56" s="49">
         <v>0.75</v>
       </c>
       <c r="E56" s="49">
-        <f t="shared" si="22"/>
-        <v>0.75</v>
-      </c>
-      <c r="F56" s="49">
         <f t="shared" si="23"/>
         <v>0.75</v>
       </c>
+      <c r="F56" s="49">
+        <f t="shared" si="24"/>
+        <v>0.75</v>
+      </c>
       <c r="G56" s="49">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.5</v>
       </c>
       <c r="H56" s="49">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.375</v>
       </c>
     </row>
@@ -42280,25 +42275,26 @@
         <v>4975</v>
       </c>
       <c r="C57" s="3">
+        <f t="shared" si="22"/>
         <v>2.0100502512562814E-4</v>
       </c>
       <c r="D57" s="5">
         <v>0.94</v>
       </c>
       <c r="E57" s="5">
-        <f t="shared" si="22"/>
-        <v>0.94</v>
-      </c>
-      <c r="F57" s="5">
         <f t="shared" si="23"/>
         <v>0.94</v>
       </c>
+      <c r="F57" s="5">
+        <f t="shared" si="24"/>
+        <v>0.94</v>
+      </c>
       <c r="G57" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.62666666666666659</v>
       </c>
       <c r="H57" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.47</v>
       </c>
     </row>
@@ -42307,62 +42303,63 @@
         <v>9975</v>
       </c>
       <c r="C58" s="3">
+        <f t="shared" si="22"/>
         <v>1.0025062656641604E-4</v>
       </c>
       <c r="D58" s="5">
         <v>1.125</v>
       </c>
       <c r="E58" s="5">
-        <f t="shared" si="22"/>
-        <v>1.125</v>
-      </c>
-      <c r="F58" s="5">
         <f t="shared" si="23"/>
         <v>1.125</v>
       </c>
+      <c r="F58" s="5">
+        <f t="shared" si="24"/>
+        <v>1.125</v>
+      </c>
       <c r="G58" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.75</v>
       </c>
       <c r="H58" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.5625</v>
       </c>
     </row>
     <row r="59" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="60" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B60" s="66" t="s">
+      <c r="B60" s="65" t="s">
         <v>91</v>
       </c>
-      <c r="C60" s="67" t="s">
+      <c r="C60" s="66" t="s">
         <v>89</v>
       </c>
-      <c r="D60" s="68" t="s">
+      <c r="D60" s="67" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="61" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B61" s="69">
+      <c r="B61" s="68">
         <v>1E-3</v>
       </c>
-      <c r="C61" s="71">
+      <c r="C61" s="70">
         <f>1/475</f>
         <v>2.1052631578947368E-3</v>
       </c>
-      <c r="D61" s="72">
+      <c r="D61" s="71">
         <f>1/2475</f>
         <v>4.0404040404040404E-4</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="70">
+      <c r="B62" s="69">
         <v>4</v>
       </c>
-      <c r="C62" s="73">
+      <c r="C62" s="72">
         <f>C61</f>
         <v>2.1052631578947368E-3</v>
       </c>
-      <c r="D62" s="74">
+      <c r="D62" s="73">
         <f>D61</f>
         <v>4.0404040404040404E-4</v>
       </c>
@@ -42403,24 +42400,24 @@
       <c r="D66" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E66" s="75">
+      <c r="E66" s="74">
         <v>1</v>
       </c>
-      <c r="F66" s="75">
+      <c r="F66" s="74">
         <f>(1/F64)</f>
         <v>1</v>
       </c>
-      <c r="G66" s="75">
-        <f t="shared" ref="G66:H66" si="26">(1/G64)</f>
+      <c r="G66" s="74">
+        <f t="shared" ref="G66:H66" si="27">(1/G64)</f>
         <v>0.66666666666666663</v>
       </c>
-      <c r="H66" s="75">
-        <f t="shared" si="26"/>
+      <c r="H66" s="74">
+        <f t="shared" si="27"/>
         <v>0.5</v>
       </c>
     </row>
     <row r="87" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B87" s="80" t="s">
+      <c r="B87" s="78" t="s">
         <v>99</v>
       </c>
     </row>
@@ -42430,7 +42427,7 @@
       </c>
     </row>
     <row r="89" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B89" s="60" t="s">
+      <c r="B89" s="59" t="s">
         <v>59</v>
       </c>
       <c r="C89" s="53">
@@ -42442,7 +42439,7 @@
       <c r="E89" s="53">
         <v>275</v>
       </c>
-      <c r="F89" s="61">
+      <c r="F89" s="60">
         <v>475</v>
       </c>
       <c r="G89" s="53">
@@ -42451,7 +42448,7 @@
       <c r="H89" s="53">
         <v>1275</v>
       </c>
-      <c r="I89" s="61">
+      <c r="I89" s="60">
         <v>2475</v>
       </c>
       <c r="J89" s="53">
@@ -42462,43 +42459,43 @@
       </c>
     </row>
     <row r="90" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="62" t="s">
+      <c r="B90" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="C90" s="63">
+      <c r="C90" s="62">
         <f>1/C89</f>
         <v>1.3333333333333334E-2</v>
       </c>
-      <c r="D90" s="63">
-        <f t="shared" ref="D90:K90" si="27">1/D89</f>
+      <c r="D90" s="62">
+        <f t="shared" ref="D90:K90" si="28">1/D89</f>
         <v>5.7142857142857143E-3</v>
       </c>
-      <c r="E90" s="63">
-        <f t="shared" si="27"/>
+      <c r="E90" s="62">
+        <f t="shared" si="28"/>
         <v>3.6363636363636364E-3</v>
       </c>
-      <c r="F90" s="64">
-        <f t="shared" si="27"/>
+      <c r="F90" s="63">
+        <f t="shared" si="28"/>
         <v>2.1052631578947368E-3</v>
       </c>
-      <c r="G90" s="63">
-        <f t="shared" si="27"/>
+      <c r="G90" s="62">
+        <f t="shared" si="28"/>
         <v>1.0256410256410256E-3</v>
       </c>
-      <c r="H90" s="63">
-        <f t="shared" si="27"/>
+      <c r="H90" s="62">
+        <f t="shared" si="28"/>
         <v>7.8431372549019605E-4</v>
       </c>
-      <c r="I90" s="64">
-        <f t="shared" si="27"/>
+      <c r="I90" s="63">
+        <f t="shared" si="28"/>
         <v>4.0404040404040404E-4</v>
       </c>
-      <c r="J90" s="63">
-        <f t="shared" si="27"/>
+      <c r="J90" s="62">
+        <f t="shared" si="28"/>
         <v>2.0100502512562814E-4</v>
       </c>
-      <c r="K90" s="65">
-        <f t="shared" si="27"/>
+      <c r="K90" s="64">
+        <f t="shared" si="28"/>
         <v>1.0025062656641604E-4</v>
       </c>
     </row>
@@ -42538,63 +42535,63 @@
       <c r="B92" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C92" s="55">
+      <c r="C92">
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="D92" s="55">
+      <c r="D92">
         <v>7.2300000000000003E-2</v>
       </c>
-      <c r="E92" s="55">
+      <c r="E92">
         <v>9.6799999999999997E-2</v>
       </c>
-      <c r="F92" s="55">
+      <c r="F92">
         <v>0.1353</v>
       </c>
-      <c r="G92" s="55">
+      <c r="G92">
         <v>0.2049</v>
       </c>
-      <c r="H92" s="55">
+      <c r="H92">
         <v>0.23699999999999999</v>
       </c>
-      <c r="I92" s="55">
+      <c r="I92">
         <v>0.33300000000000002</v>
       </c>
-      <c r="J92" s="55">
+      <c r="J92">
         <v>0.46029999999999999</v>
       </c>
-      <c r="K92" s="56">
+      <c r="K92" s="55">
         <v>0.61229999999999996</v>
       </c>
     </row>
     <row r="93" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="57" t="s">
+      <c r="B93" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="C93" s="58">
+      <c r="C93" s="57">
         <v>7.6499999999999999E-2</v>
       </c>
-      <c r="D93" s="58">
+      <c r="D93" s="57">
         <v>0.13089999999999999</v>
       </c>
-      <c r="E93" s="58">
+      <c r="E93" s="57">
         <v>0.1736</v>
       </c>
-      <c r="F93" s="58">
+      <c r="F93" s="57">
         <v>0.2392</v>
       </c>
-      <c r="G93" s="58">
+      <c r="G93" s="57">
         <v>0.34949999999999998</v>
       </c>
-      <c r="H93" s="58">
+      <c r="H93" s="57">
         <v>0.39689999999999998</v>
       </c>
-      <c r="I93" s="58">
+      <c r="I93" s="57">
         <v>0.52990000000000004</v>
       </c>
-      <c r="J93" s="58">
+      <c r="J93" s="57">
         <v>0.69689999999999996</v>
       </c>
-      <c r="K93" s="59">
+      <c r="K93" s="58">
         <v>0.89090000000000003</v>
       </c>
     </row>
@@ -42604,7 +42601,7 @@
       </c>
     </row>
     <row r="97" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B97" s="57" t="s">
+      <c r="B97" s="56" t="s">
         <v>58</v>
       </c>
       <c r="C97">
@@ -42641,7 +42638,7 @@
       </c>
     </row>
     <row r="100" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="57" t="s">
+      <c r="B100" s="56" t="s">
         <v>58</v>
       </c>
       <c r="C100">
@@ -42678,7 +42675,7 @@
       </c>
     </row>
     <row r="103" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B103" s="57" t="s">
+      <c r="B103" s="56" t="s">
         <v>58</v>
       </c>
       <c r="C103">
@@ -42720,7 +42717,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
@@ -42738,7 +42735,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="10" t="s">
         <v>101</v>
       </c>
       <c r="B1" s="50" t="s">
@@ -44190,118 +44187,118 @@
       </c>
       <c r="C20" s="46"/>
     </row>
-    <row r="21" spans="1:29" s="90" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="87" t="s">
+    <row r="21" spans="1:29" s="87" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="B21" s="89" t="s">
+      <c r="B21" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="91" t="str">
+      <c r="C21" s="88" t="str">
         <f>"ln(λ_im("&amp;C1&amp;"))"</f>
         <v>ln(λ_im(T=0.01s))</v>
       </c>
-      <c r="D21" s="91" t="str">
+      <c r="D21" s="88" t="str">
         <f t="shared" ref="D21:AC21" si="1">"ln(λ_im("&amp;D1&amp;"))"</f>
         <v>ln(λ_im(T=0.015s))</v>
       </c>
-      <c r="E21" s="91" t="str">
+      <c r="E21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.02s))</v>
       </c>
-      <c r="F21" s="91" t="str">
+      <c r="F21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.03s))</v>
       </c>
-      <c r="G21" s="91" t="str">
+      <c r="G21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.04s))</v>
       </c>
-      <c r="H21" s="91" t="str">
+      <c r="H21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.05s))</v>
       </c>
-      <c r="I21" s="91" t="str">
+      <c r="I21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.06s))</v>
       </c>
-      <c r="J21" s="91" t="str">
+      <c r="J21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.075s))</v>
       </c>
-      <c r="K21" s="91" t="str">
+      <c r="K21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.09s))</v>
       </c>
-      <c r="L21" s="91" t="str">
+      <c r="L21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.1s))</v>
       </c>
-      <c r="M21" s="91" t="str">
+      <c r="M21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.15s))</v>
       </c>
-      <c r="N21" s="91" t="str">
+      <c r="N21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.2s))</v>
       </c>
-      <c r="O21" s="91" t="str">
+      <c r="O21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.3s))</v>
       </c>
-      <c r="P21" s="91" t="str">
+      <c r="P21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.4s))</v>
       </c>
-      <c r="Q21" s="91" t="str">
+      <c r="Q21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.5s))</v>
       </c>
-      <c r="R21" s="91" t="str">
+      <c r="R21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.6s))</v>
       </c>
-      <c r="S21" s="91" t="str">
+      <c r="S21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.7s))</v>
       </c>
-      <c r="T21" s="91" t="str">
+      <c r="T21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.75s))</v>
       </c>
-      <c r="U21" s="91" t="str">
+      <c r="U21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.8s))</v>
       </c>
-      <c r="V21" s="91" t="str">
+      <c r="V21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=0.9s))</v>
       </c>
-      <c r="W21" s="91" t="str">
+      <c r="W21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=1s))</v>
       </c>
-      <c r="X21" s="91" t="str">
+      <c r="X21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=1.2s))</v>
       </c>
-      <c r="Y21" s="91" t="str">
+      <c r="Y21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=1.5s))</v>
       </c>
-      <c r="Z21" s="91" t="str">
+      <c r="Z21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=2s))</v>
       </c>
-      <c r="AA21" s="91" t="str">
+      <c r="AA21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=2.5s))</v>
       </c>
-      <c r="AB21" s="91" t="str">
+      <c r="AB21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=3s))</v>
       </c>
-      <c r="AC21" s="91" t="str">
+      <c r="AC21" s="88" t="str">
         <f t="shared" si="1"/>
         <v>ln(λ_im(T=5s))</v>
       </c>
@@ -46061,118 +46058,118 @@
         <v>-18.128931705678902</v>
       </c>
     </row>
-    <row r="39" spans="1:29" s="94" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="93" t="str">
+    <row r="39" spans="1:29" s="91" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="90" t="str">
         <f>"Sa("&amp;C1&amp;")"</f>
         <v>Sa(T=0.01s)</v>
       </c>
-      <c r="D39" s="93" t="str">
+      <c r="D39" s="90" t="str">
         <f t="shared" ref="D39:AC39" si="19">"Sa("&amp;D1&amp;")"</f>
         <v>Sa(T=0.015s)</v>
       </c>
-      <c r="E39" s="93" t="str">
+      <c r="E39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.02s)</v>
       </c>
-      <c r="F39" s="93" t="str">
+      <c r="F39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.03s)</v>
       </c>
-      <c r="G39" s="93" t="str">
+      <c r="G39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.04s)</v>
       </c>
-      <c r="H39" s="93" t="str">
+      <c r="H39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.05s)</v>
       </c>
-      <c r="I39" s="93" t="str">
+      <c r="I39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.06s)</v>
       </c>
-      <c r="J39" s="93" t="str">
+      <c r="J39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.075s)</v>
       </c>
-      <c r="K39" s="93" t="str">
+      <c r="K39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.09s)</v>
       </c>
-      <c r="L39" s="93" t="str">
+      <c r="L39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.1s)</v>
       </c>
-      <c r="M39" s="93" t="str">
+      <c r="M39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.15s)</v>
       </c>
-      <c r="N39" s="93" t="str">
+      <c r="N39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.2s)</v>
       </c>
-      <c r="O39" s="93" t="str">
+      <c r="O39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.3s)</v>
       </c>
-      <c r="P39" s="93" t="str">
+      <c r="P39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.4s)</v>
       </c>
-      <c r="Q39" s="93" t="str">
+      <c r="Q39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.5s)</v>
       </c>
-      <c r="R39" s="93" t="str">
+      <c r="R39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.6s)</v>
       </c>
-      <c r="S39" s="93" t="str">
+      <c r="S39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.7s)</v>
       </c>
-      <c r="T39" s="93" t="str">
+      <c r="T39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.75s)</v>
       </c>
-      <c r="U39" s="93" t="str">
+      <c r="U39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.8s)</v>
       </c>
-      <c r="V39" s="93" t="str">
+      <c r="V39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=0.9s)</v>
       </c>
-      <c r="W39" s="93" t="str">
+      <c r="W39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=1s)</v>
       </c>
-      <c r="X39" s="93" t="str">
+      <c r="X39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=1.2s)</v>
       </c>
-      <c r="Y39" s="93" t="str">
+      <c r="Y39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=1.5s)</v>
       </c>
-      <c r="Z39" s="93" t="str">
+      <c r="Z39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=2s)</v>
       </c>
-      <c r="AA39" s="93" t="str">
+      <c r="AA39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=2.5s)</v>
       </c>
-      <c r="AB39" s="93" t="str">
+      <c r="AB39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=3s)</v>
       </c>
-      <c r="AC39" s="93" t="str">
+      <c r="AC39" s="90" t="str">
         <f t="shared" si="19"/>
         <v>Sa(T=5s)</v>
       </c>
     </row>
     <row r="40" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="92" t="s">
+      <c r="A40" s="89" t="s">
         <v>106</v>
       </c>
       <c r="C40">
@@ -46285,7 +46282,7 @@
       </c>
     </row>
     <row r="41" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="92" t="s">
+      <c r="A41" s="89" t="s">
         <v>105</v>
       </c>
       <c r="C41">
@@ -46398,52 +46395,52 @@
       </c>
     </row>
     <row r="43" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="83" t="s">
+      <c r="A43" s="80" t="s">
         <v>103</v>
       </c>
-      <c r="C43" s="85">
+      <c r="C43" s="82">
         <f ca="1">(E53-C40)/C40</f>
         <v>-0.18391328043920424</v>
       </c>
-      <c r="W43" s="85">
+      <c r="W43" s="82">
         <f ca="1">(F53-W40)/W40</f>
         <v>0.3412821076387717</v>
       </c>
-      <c r="Y43" s="85">
+      <c r="Y43" s="82">
         <f ca="1">(G53-Y40)/Y40</f>
         <v>0.38503787474896811</v>
       </c>
-      <c r="Z43" s="85">
+      <c r="Z43" s="82">
         <f ca="1">(H53-Z40)/Z40</f>
         <v>0.46809249694456884</v>
       </c>
     </row>
     <row r="44" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="83" t="s">
+      <c r="A44" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="C44" s="85">
+      <c r="C44" s="82">
         <f ca="1">(E56-C41)/C41</f>
         <v>-0.48702120406753541</v>
       </c>
-      <c r="W44" s="85">
+      <c r="W44" s="82">
         <f ca="1">(F56-W41)/W41</f>
         <v>-0.23536490654239753</v>
       </c>
-      <c r="Y44" s="85">
+      <c r="Y44" s="82">
         <f ca="1">(G56-Y41)/Y41</f>
         <v>-0.19821388491704026</v>
       </c>
-      <c r="Z44" s="85">
+      <c r="Z44" s="82">
         <f ca="1">(H56-Z41)/Z41</f>
         <v>-0.16834903109514873</v>
       </c>
     </row>
     <row r="45" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="83"/>
+      <c r="A45" s="80"/>
     </row>
     <row r="46" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="83"/>
+      <c r="A46" s="80"/>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B48" s="46" t="s">
@@ -46451,36 +46448,36 @@
       </c>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B49" s="76" t="s">
+      <c r="B49" s="75" t="s">
         <v>39</v>
       </c>
-      <c r="C49" s="76" t="s">
+      <c r="C49" s="75" t="s">
         <v>44</v>
       </c>
-      <c r="D49" s="76" t="s">
+      <c r="D49" s="75" t="s">
         <v>98</v>
       </c>
-      <c r="E49" s="109" t="s">
+      <c r="E49" s="106" t="s">
         <v>41</v>
       </c>
-      <c r="F49" s="110"/>
-      <c r="G49" s="110"/>
-      <c r="H49" s="110"/>
+      <c r="F49" s="107"/>
+      <c r="G49" s="107"/>
+      <c r="H49" s="107"/>
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="47"/>
       <c r="C50" s="47"/>
       <c r="D50" s="47"/>
-      <c r="E50" s="76" t="s">
+      <c r="E50" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="F50" s="76" t="s">
+      <c r="F50" s="75" t="s">
         <v>40</v>
       </c>
-      <c r="G50" s="76" t="s">
+      <c r="G50" s="75" t="s">
         <v>92</v>
       </c>
-      <c r="H50" s="76" t="s">
+      <c r="H50" s="75" t="s">
         <v>93</v>
       </c>
     </row>
@@ -46489,25 +46486,26 @@
         <v>175</v>
       </c>
       <c r="C51" s="3">
+        <f t="shared" ref="C51:C58" si="22">1/B51</f>
         <v>5.7142857142857143E-3</v>
       </c>
       <c r="D51" s="5">
         <v>0.17499999999999999</v>
       </c>
       <c r="E51" s="5">
-        <f t="shared" ref="E51:E58" si="22">(D51*$E$68)</f>
+        <f t="shared" ref="E51:E58" si="23">(D51*$E$68)</f>
         <v>0.17499999999999999</v>
       </c>
       <c r="F51" s="5">
-        <f t="shared" ref="F51:F58" si="23">(D51*$F$68)</f>
+        <f t="shared" ref="F51:F58" si="24">(D51*$F$68)</f>
         <v>0.17499999999999999</v>
       </c>
       <c r="G51" s="5">
-        <f t="shared" ref="G51:G58" si="24">(D51*$G$68)</f>
+        <f t="shared" ref="G51:G58" si="25">(D51*$G$68)</f>
         <v>0.11666666666666665</v>
       </c>
       <c r="H51" s="5">
-        <f t="shared" ref="H51:H58" si="25">(D51*$H$68)</f>
+        <f t="shared" ref="H51:H58" si="26">(D51*$H$68)</f>
         <v>8.7499999999999994E-2</v>
       </c>
     </row>
@@ -46516,25 +46514,26 @@
         <v>275</v>
       </c>
       <c r="C52" s="3">
+        <f t="shared" si="22"/>
         <v>3.6363636363636364E-3</v>
       </c>
       <c r="D52" s="5">
         <v>0.21</v>
       </c>
       <c r="E52" s="5">
-        <f t="shared" si="22"/>
-        <v>0.21</v>
-      </c>
-      <c r="F52" s="5">
         <f t="shared" si="23"/>
         <v>0.21</v>
       </c>
+      <c r="F52" s="5">
+        <f t="shared" si="24"/>
+        <v>0.21</v>
+      </c>
       <c r="G52" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.13999999999999999</v>
       </c>
       <c r="H52" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.105</v>
       </c>
     </row>
@@ -46543,25 +46542,26 @@
         <v>475</v>
       </c>
       <c r="C53" s="48">
+        <f t="shared" si="22"/>
         <v>2.1052631578947368E-3</v>
       </c>
       <c r="D53" s="49">
         <v>0.23300000000000001</v>
       </c>
       <c r="E53" s="49">
-        <f t="shared" si="22"/>
-        <v>0.23300000000000001</v>
-      </c>
-      <c r="F53" s="49">
         <f t="shared" si="23"/>
         <v>0.23300000000000001</v>
       </c>
+      <c r="F53" s="49">
+        <f t="shared" si="24"/>
+        <v>0.23300000000000001</v>
+      </c>
       <c r="G53" s="49">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.15533333333333332</v>
       </c>
       <c r="H53" s="49">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.11650000000000001</v>
       </c>
     </row>
@@ -46570,25 +46570,26 @@
         <v>975</v>
       </c>
       <c r="C54" s="3">
+        <f t="shared" si="22"/>
         <v>1.0256410256410256E-3</v>
       </c>
       <c r="D54" s="5">
         <v>0.28000000000000003</v>
       </c>
       <c r="E54" s="5">
-        <f t="shared" si="22"/>
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="F54" s="5">
         <f t="shared" si="23"/>
         <v>0.28000000000000003</v>
       </c>
+      <c r="F54" s="5">
+        <f t="shared" si="24"/>
+        <v>0.28000000000000003</v>
+      </c>
       <c r="G54" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.18666666666666668</v>
       </c>
       <c r="H54" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.14000000000000001</v>
       </c>
     </row>
@@ -46597,25 +46598,26 @@
         <v>1275</v>
       </c>
       <c r="C55" s="3">
+        <f t="shared" si="22"/>
         <v>7.8431372549019605E-4</v>
       </c>
       <c r="D55" s="5">
         <v>0.29170000000000001</v>
       </c>
       <c r="E55" s="5">
-        <f t="shared" si="22"/>
-        <v>0.29170000000000001</v>
-      </c>
-      <c r="F55" s="5">
         <f t="shared" si="23"/>
         <v>0.29170000000000001</v>
       </c>
+      <c r="F55" s="5">
+        <f t="shared" si="24"/>
+        <v>0.29170000000000001</v>
+      </c>
       <c r="G55" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.19446666666666668</v>
       </c>
       <c r="H55" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.14585000000000001</v>
       </c>
     </row>
@@ -46624,25 +46626,26 @@
         <v>2475</v>
       </c>
       <c r="C56" s="48">
+        <f t="shared" si="22"/>
         <v>4.0404040404040404E-4</v>
       </c>
       <c r="D56" s="49">
         <v>0.35</v>
       </c>
       <c r="E56" s="49">
-        <f t="shared" si="22"/>
-        <v>0.35</v>
-      </c>
-      <c r="F56" s="49">
         <f t="shared" si="23"/>
         <v>0.35</v>
       </c>
+      <c r="F56" s="49">
+        <f t="shared" si="24"/>
+        <v>0.35</v>
+      </c>
       <c r="G56" s="49">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.23333333333333331</v>
       </c>
       <c r="H56" s="49">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.17499999999999999</v>
       </c>
     </row>
@@ -46651,25 +46654,26 @@
         <v>4975</v>
       </c>
       <c r="C57" s="3">
+        <f t="shared" si="22"/>
         <v>2.0100502512562814E-4</v>
       </c>
       <c r="D57" s="5">
         <v>0.44</v>
       </c>
       <c r="E57" s="5">
-        <f t="shared" si="22"/>
-        <v>0.44</v>
-      </c>
-      <c r="F57" s="5">
         <f t="shared" si="23"/>
         <v>0.44</v>
       </c>
+      <c r="F57" s="5">
+        <f t="shared" si="24"/>
+        <v>0.44</v>
+      </c>
       <c r="G57" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.29333333333333333</v>
       </c>
       <c r="H57" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.22</v>
       </c>
     </row>
@@ -46678,25 +46682,26 @@
         <v>9975</v>
       </c>
       <c r="C58" s="3">
+        <f t="shared" si="22"/>
         <v>1.0025062656641604E-4</v>
       </c>
       <c r="D58" s="5">
         <v>0.52500000000000002</v>
       </c>
       <c r="E58" s="5">
-        <f t="shared" si="22"/>
-        <v>0.52500000000000002</v>
-      </c>
-      <c r="F58" s="5">
         <f t="shared" si="23"/>
         <v>0.52500000000000002</v>
       </c>
+      <c r="F58" s="5">
+        <f t="shared" si="24"/>
+        <v>0.52500000000000002</v>
+      </c>
       <c r="G58" s="5">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.35</v>
       </c>
       <c r="H58" s="5">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.26250000000000001</v>
       </c>
     </row>
@@ -46720,46 +46725,46 @@
     </row>
     <row r="61" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="62" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B62" s="66" t="s">
+      <c r="B62" s="65" t="s">
         <v>91</v>
       </c>
-      <c r="C62" s="67" t="s">
+      <c r="C62" s="66" t="s">
         <v>89</v>
       </c>
-      <c r="D62" s="68" t="s">
+      <c r="D62" s="67" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="63" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B63" s="69">
+      <c r="B63" s="68">
         <v>1E-3</v>
       </c>
-      <c r="C63" s="71">
+      <c r="C63" s="70">
         <f>1/475</f>
         <v>2.1052631578947368E-3</v>
       </c>
-      <c r="D63" s="72">
+      <c r="D63" s="71">
         <f>1/2475</f>
         <v>4.0404040404040404E-4</v>
       </c>
     </row>
     <row r="64" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="70">
+      <c r="B64" s="69">
         <v>4</v>
       </c>
-      <c r="C64" s="73">
+      <c r="C64" s="72">
         <f>C63</f>
         <v>2.1052631578947368E-3</v>
       </c>
-      <c r="D64" s="74">
+      <c r="D64" s="73">
         <f>D63</f>
         <v>4.0404040404040404E-4</v>
       </c>
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B65" s="79"/>
-      <c r="C65" s="71"/>
-      <c r="D65" s="71"/>
+      <c r="B65" s="29"/>
+      <c r="C65" s="70"/>
+      <c r="D65" s="70"/>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D66" s="3" t="s">
@@ -46803,17 +46808,17 @@
       <c r="F68" s="3">
         <v>1</v>
       </c>
-      <c r="G68" s="75">
+      <c r="G68" s="74">
         <f>(1/G66)</f>
         <v>0.66666666666666663</v>
       </c>
-      <c r="H68" s="75">
+      <c r="H68" s="74">
         <f>(1/H66)</f>
         <v>0.5</v>
       </c>
     </row>
     <row r="72" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B72" s="80" t="s">
+      <c r="B72" s="78" t="s">
         <v>99</v>
       </c>
     </row>
@@ -46823,7 +46828,7 @@
       </c>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B74" s="60" t="s">
+      <c r="B74" s="59" t="s">
         <v>59</v>
       </c>
       <c r="C74" s="53">
@@ -46835,7 +46840,7 @@
       <c r="E74" s="53">
         <v>275</v>
       </c>
-      <c r="F74" s="61">
+      <c r="F74" s="60">
         <v>475</v>
       </c>
       <c r="G74" s="53">
@@ -46844,7 +46849,7 @@
       <c r="H74" s="53">
         <v>1275</v>
       </c>
-      <c r="I74" s="61">
+      <c r="I74" s="60">
         <v>2475</v>
       </c>
       <c r="J74" s="53">
@@ -46855,43 +46860,43 @@
       </c>
     </row>
     <row r="75" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="62" t="s">
+      <c r="B75" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="C75" s="63">
+      <c r="C75" s="62">
         <f>1/C74</f>
         <v>1.3333333333333334E-2</v>
       </c>
-      <c r="D75" s="63">
-        <f t="shared" ref="D75:K75" si="26">1/D74</f>
+      <c r="D75" s="62">
+        <f t="shared" ref="D75:K75" si="27">1/D74</f>
         <v>5.7142857142857143E-3</v>
       </c>
-      <c r="E75" s="63">
-        <f t="shared" si="26"/>
+      <c r="E75" s="62">
+        <f t="shared" si="27"/>
         <v>3.6363636363636364E-3</v>
       </c>
-      <c r="F75" s="64">
-        <f t="shared" si="26"/>
+      <c r="F75" s="63">
+        <f t="shared" si="27"/>
         <v>2.1052631578947368E-3</v>
       </c>
-      <c r="G75" s="63">
-        <f t="shared" si="26"/>
+      <c r="G75" s="62">
+        <f t="shared" si="27"/>
         <v>1.0256410256410256E-3</v>
       </c>
-      <c r="H75" s="63">
-        <f t="shared" si="26"/>
+      <c r="H75" s="62">
+        <f t="shared" si="27"/>
         <v>7.8431372549019605E-4</v>
       </c>
-      <c r="I75" s="64">
-        <f t="shared" si="26"/>
+      <c r="I75" s="63">
+        <f t="shared" si="27"/>
         <v>4.0404040404040404E-4</v>
       </c>
-      <c r="J75" s="63">
-        <f t="shared" si="26"/>
+      <c r="J75" s="62">
+        <f t="shared" si="27"/>
         <v>2.0100502512562814E-4</v>
       </c>
-      <c r="K75" s="65">
-        <f t="shared" si="26"/>
+      <c r="K75" s="64">
+        <f t="shared" si="27"/>
         <v>1.0025062656641604E-4</v>
       </c>
     </row>
@@ -46931,76 +46936,76 @@
       <c r="B77" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C77" s="55">
+      <c r="C77">
         <v>4.0500000000000001E-2</v>
       </c>
-      <c r="D77" s="55">
+      <c r="D77">
         <v>7.2300000000000003E-2</v>
       </c>
-      <c r="E77" s="55">
+      <c r="E77">
         <v>9.6799999999999997E-2</v>
       </c>
-      <c r="F77" s="55">
+      <c r="F77">
         <v>0.1353</v>
       </c>
-      <c r="G77" s="55">
+      <c r="G77">
         <v>0.2049</v>
       </c>
-      <c r="H77" s="55">
+      <c r="H77">
         <v>0.23699999999999999</v>
       </c>
-      <c r="I77" s="55">
+      <c r="I77">
         <v>0.33300000000000002</v>
       </c>
-      <c r="J77" s="55">
+      <c r="J77">
         <v>0.46029999999999999</v>
       </c>
-      <c r="K77" s="56">
+      <c r="K77" s="55">
         <v>0.61229999999999996</v>
       </c>
     </row>
     <row r="78" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="57" t="s">
+      <c r="B78" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="C78" s="58">
+      <c r="C78" s="57">
         <v>7.6499999999999999E-2</v>
       </c>
-      <c r="D78" s="58">
+      <c r="D78" s="57">
         <v>0.13089999999999999</v>
       </c>
-      <c r="E78" s="58">
+      <c r="E78" s="57">
         <v>0.1736</v>
       </c>
-      <c r="F78" s="58">
+      <c r="F78" s="57">
         <v>0.2392</v>
       </c>
-      <c r="G78" s="58">
+      <c r="G78" s="57">
         <v>0.34949999999999998</v>
       </c>
-      <c r="H78" s="58">
+      <c r="H78" s="57">
         <v>0.39689999999999998</v>
       </c>
-      <c r="I78" s="58">
+      <c r="I78" s="57">
         <v>0.52990000000000004</v>
       </c>
-      <c r="J78" s="58">
+      <c r="J78" s="57">
         <v>0.69689999999999996</v>
       </c>
-      <c r="K78" s="59">
+      <c r="K78" s="58">
         <v>0.89090000000000003</v>
       </c>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C80" s="78"/>
-      <c r="D80" s="78"/>
-      <c r="E80" s="78"/>
-      <c r="F80" s="78"/>
-      <c r="G80" s="78"/>
-      <c r="H80" s="78"/>
-      <c r="I80" s="78"/>
-      <c r="J80" s="78"/>
-      <c r="K80" s="78"/>
+      <c r="C80" s="77"/>
+      <c r="D80" s="77"/>
+      <c r="E80" s="77"/>
+      <c r="F80" s="77"/>
+      <c r="G80" s="77"/>
+      <c r="H80" s="77"/>
+      <c r="I80" s="77"/>
+      <c r="J80" s="77"/>
+      <c r="K80" s="77"/>
     </row>
     <row r="81" spans="2:11" ht="21" x14ac:dyDescent="0.35">
       <c r="B81" s="52" t="s">
@@ -47011,31 +47016,31 @@
       <c r="B82" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C82" s="77">
+      <c r="C82" s="76">
         <v>3.0534253552491002E-2</v>
       </c>
-      <c r="D82" s="77">
+      <c r="D82" s="76">
         <v>5.2247799204166001E-2</v>
       </c>
-      <c r="E82" s="77">
+      <c r="E82" s="76">
         <v>6.8864213966061003E-2</v>
       </c>
-      <c r="F82" s="77">
+      <c r="F82" s="76">
         <v>9.4689758228719001E-2</v>
       </c>
-      <c r="G82" s="77">
+      <c r="G82" s="76">
         <v>0.14097016526665701</v>
       </c>
-      <c r="H82" s="77">
+      <c r="H82" s="76">
         <v>0.162832985239144</v>
       </c>
-      <c r="I82" s="77">
+      <c r="I82" s="76">
         <v>0.23135077772705301</v>
       </c>
-      <c r="J82" s="77">
+      <c r="J82" s="76">
         <v>0.332024386493319</v>
       </c>
-      <c r="K82" s="77">
+      <c r="K82" s="76">
         <v>0.47259360336538903</v>
       </c>
     </row>
@@ -47048,31 +47053,31 @@
       <c r="B85" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C85" s="77">
+      <c r="C85" s="76">
         <v>2.6119697499103998E-2</v>
       </c>
-      <c r="D85" s="77">
+      <c r="D85" s="76">
         <v>4.4263655745839001E-2</v>
       </c>
-      <c r="E85" s="77">
+      <c r="E85" s="76">
         <v>5.7840751599430001E-2</v>
       </c>
-      <c r="F85" s="77">
+      <c r="F85" s="76">
         <v>7.9059267015249998E-2</v>
       </c>
-      <c r="G85" s="77">
+      <c r="G85" s="76">
         <v>0.116949276929855</v>
       </c>
-      <c r="H85" s="77">
+      <c r="H85" s="76">
         <v>0.13521223795982901</v>
       </c>
-      <c r="I85" s="77">
+      <c r="I85" s="76">
         <v>0.194528978104341</v>
       </c>
-      <c r="J85" s="77">
+      <c r="J85" s="76">
         <v>0.28896669111729101</v>
       </c>
-      <c r="K85" s="77">
+      <c r="K85" s="76">
         <v>0.43849156574250803</v>
       </c>
     </row>
@@ -47085,31 +47090,31 @@
       <c r="B88" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C88" s="77">
+      <c r="C88" s="76">
         <v>2.6119697499103998E-2</v>
       </c>
-      <c r="D88" s="77">
+      <c r="D88" s="76">
         <v>4.4263655745839001E-2</v>
       </c>
-      <c r="E88" s="77">
+      <c r="E88" s="76">
         <v>5.7840751599430001E-2</v>
       </c>
-      <c r="F88" s="77">
+      <c r="F88" s="76">
         <v>7.9059267015249998E-2</v>
       </c>
-      <c r="G88" s="77">
+      <c r="G88" s="76">
         <v>0.116949276929855</v>
       </c>
-      <c r="H88" s="77">
+      <c r="H88" s="76">
         <v>0.13521223795982901</v>
       </c>
-      <c r="I88" s="77">
+      <c r="I88" s="76">
         <v>0.194528978104341</v>
       </c>
-      <c r="J88" s="77">
+      <c r="J88" s="76">
         <v>0.28896669111729101</v>
       </c>
-      <c r="K88" s="77">
+      <c r="K88" s="76">
         <v>0.43849156574250803</v>
       </c>
     </row>

</xml_diff>